<commit_message>
Updated the coding and finalized the matrices.
</commit_message>
<xml_diff>
--- a/Immigration_Networks/MigrationData/Matrices/DifferenceMatrices_1990.xlsx
+++ b/Immigration_Networks/MigrationData/Matrices/DifferenceMatrices_1990.xlsx
@@ -587,7 +587,7 @@
         <v>31303</v>
       </c>
       <c r="S3" t="n">
-        <v>10581</v>
+        <v>0</v>
       </c>
       <c r="T3" t="n">
         <v>2224</v>
@@ -649,7 +649,7 @@
         <v>82489</v>
       </c>
       <c r="S4" t="n">
-        <v>427</v>
+        <v>10581</v>
       </c>
       <c r="T4" t="n">
         <v>4323</v>
@@ -711,7 +711,7 @@
         <v>744830</v>
       </c>
       <c r="S5" t="n">
-        <v>1161</v>
+        <v>427</v>
       </c>
       <c r="T5" t="n">
         <v>981</v>
@@ -773,7 +773,7 @@
         <v>55681</v>
       </c>
       <c r="S6" t="n">
-        <v>0</v>
+        <v>1161</v>
       </c>
       <c r="T6" t="n">
         <v>22198</v>
@@ -1838,7 +1838,7 @@
         <v>28225</v>
       </c>
       <c r="S3" t="n">
-        <v>10179</v>
+        <v>-402</v>
       </c>
       <c r="T3" t="n">
         <v>1855</v>
@@ -1900,7 +1900,7 @@
         <v>70683</v>
       </c>
       <c r="S4" t="n">
-        <v>-22936</v>
+        <v>-12782</v>
       </c>
       <c r="T4" t="n">
         <v>3103</v>
@@ -1962,7 +1962,7 @@
         <v>505832</v>
       </c>
       <c r="S5" t="n">
-        <v>-3872</v>
+        <v>-4606</v>
       </c>
       <c r="T5" t="n">
         <v>-2358</v>
@@ -2024,7 +2024,7 @@
         <v>50031</v>
       </c>
       <c r="S6" t="n">
-        <v>-1393</v>
+        <v>-232</v>
       </c>
       <c r="T6" t="n">
         <v>19849</v>
@@ -2782,16 +2782,16 @@
         <v>122347</v>
       </c>
       <c r="C19" t="n">
-        <v>-10179</v>
+        <v>402</v>
       </c>
       <c r="D19" t="n">
-        <v>22936</v>
+        <v>12782</v>
       </c>
       <c r="E19" t="n">
-        <v>3872</v>
+        <v>4606</v>
       </c>
       <c r="F19" t="n">
-        <v>1393</v>
+        <v>232</v>
       </c>
       <c r="G19" t="n">
         <v>360</v>
@@ -3089,7 +3089,7 @@
         <v>28225</v>
       </c>
       <c r="S3" t="n">
-        <v>10179</v>
+        <v>0</v>
       </c>
       <c r="T3" t="n">
         <v>1855</v>
@@ -4033,16 +4033,16 @@
         <v>122347</v>
       </c>
       <c r="C19" t="n">
-        <v>0</v>
+        <v>402</v>
       </c>
       <c r="D19" t="n">
-        <v>22936</v>
+        <v>12782</v>
       </c>
       <c r="E19" t="n">
-        <v>3872</v>
+        <v>4606</v>
       </c>
       <c r="F19" t="n">
-        <v>1393</v>
+        <v>232</v>
       </c>
       <c r="G19" t="n">
         <v>360</v>
@@ -4340,7 +4340,7 @@
         <v>0.000113485643571536</v>
       </c>
       <c r="S3" t="n">
-        <v>0.00326562746630427</v>
+        <v>-0.000128969667104265</v>
       </c>
       <c r="T3" t="n">
         <v>0.0000939212971933633</v>
@@ -4402,7 +4402,7 @@
         <v>0.000284198609196347</v>
       </c>
       <c r="S4" t="n">
-        <v>-0.00735832906642644</v>
+        <v>-0.00410072210180776</v>
       </c>
       <c r="T4" t="n">
         <v>0.000157109318162268</v>
@@ -4464,7 +4464,7 @@
         <v>0.00203382356276624</v>
       </c>
       <c r="S5" t="n">
-        <v>-0.00124221530106397</v>
+        <v>-0.00147769723055285</v>
       </c>
       <c r="T5" t="n">
         <v>-0.000119388905003747</v>
@@ -4526,7 +4526,7 @@
         <v>0.000201162098619221</v>
       </c>
       <c r="S6" t="n">
-        <v>-0.000446902353920999</v>
+        <v>-0.0000744302556422625</v>
       </c>
       <c r="T6" t="n">
         <v>0.00100498319568252</v>
@@ -5284,16 +5284,16 @@
         <v>0.00373511336888927</v>
       </c>
       <c r="C19" t="n">
-        <v>-0.00143443110975138</v>
+        <v>0.000056650093930647</v>
       </c>
       <c r="D19" t="n">
-        <v>0.00015378506336825</v>
+        <v>0.0000857028548994144</v>
       </c>
       <c r="E19" t="n">
-        <v>0.000139333492194626</v>
+        <v>0.000165746401097222</v>
       </c>
       <c r="F19" t="n">
-        <v>0.00010366761587405</v>
+        <v>0.0000172655325791669</v>
       </c>
       <c r="G19" t="n">
         <v>0.000011097387342098</v>
@@ -5591,7 +5591,7 @@
         <v>0.113485643571536</v>
       </c>
       <c r="S3" t="n">
-        <v>3.26562746630427</v>
+        <v>-0.128969667104265</v>
       </c>
       <c r="T3" t="n">
         <v>0.0939212971933633</v>
@@ -5653,7 +5653,7 @@
         <v>0.284198609196347</v>
       </c>
       <c r="S4" t="n">
-        <v>-7.35832906642644</v>
+        <v>-4.10072210180776</v>
       </c>
       <c r="T4" t="n">
         <v>0.157109318162268</v>
@@ -5715,7 +5715,7 @@
         <v>2.03382356276624</v>
       </c>
       <c r="S5" t="n">
-        <v>-1.24221530106397</v>
+        <v>-1.47769723055285</v>
       </c>
       <c r="T5" t="n">
         <v>-0.119388905003747</v>
@@ -5777,7 +5777,7 @@
         <v>0.201162098619221</v>
       </c>
       <c r="S6" t="n">
-        <v>-0.446902353920999</v>
+        <v>-0.0744302556422625</v>
       </c>
       <c r="T6" t="n">
         <v>1.00498319568252</v>
@@ -6535,16 +6535,16 @@
         <v>3.73511336888927</v>
       </c>
       <c r="C19" t="n">
-        <v>-1.43443110975138</v>
+        <v>0.056650093930647</v>
       </c>
       <c r="D19" t="n">
-        <v>0.15378506336825</v>
+        <v>0.0857028548994144</v>
       </c>
       <c r="E19" t="n">
-        <v>0.139333492194626</v>
+        <v>0.165746401097222</v>
       </c>
       <c r="F19" t="n">
-        <v>0.10366761587405</v>
+        <v>0.0172655325791669</v>
       </c>
       <c r="G19" t="n">
         <v>0.011097387342098</v>
@@ -6842,7 +6842,7 @@
         <v>0.000113485643571536</v>
       </c>
       <c r="S3" t="n">
-        <v>0.00326562746630427</v>
+        <v>0</v>
       </c>
       <c r="T3" t="n">
         <v>0.0000939212971933633</v>
@@ -7786,16 +7786,16 @@
         <v>0.00373511336888927</v>
       </c>
       <c r="C19" t="n">
-        <v>0</v>
+        <v>0.000056650093930647</v>
       </c>
       <c r="D19" t="n">
-        <v>0.00015378506336825</v>
+        <v>0.0000857028548994144</v>
       </c>
       <c r="E19" t="n">
-        <v>0.000139333492194626</v>
+        <v>0.000165746401097222</v>
       </c>
       <c r="F19" t="n">
-        <v>0.00010366761587405</v>
+        <v>0.0000172655325791669</v>
       </c>
       <c r="G19" t="n">
         <v>0.000011097387342098</v>
@@ -8093,7 +8093,7 @@
         <v>0.113485643571536</v>
       </c>
       <c r="S3" t="n">
-        <v>3.26562746630427</v>
+        <v>0</v>
       </c>
       <c r="T3" t="n">
         <v>0.0939212971933633</v>
@@ -9037,16 +9037,16 @@
         <v>3.73511336888927</v>
       </c>
       <c r="C19" t="n">
-        <v>0</v>
+        <v>0.056650093930647</v>
       </c>
       <c r="D19" t="n">
-        <v>0.15378506336825</v>
+        <v>0.0857028548994144</v>
       </c>
       <c r="E19" t="n">
-        <v>0.139333492194626</v>
+        <v>0.165746401097222</v>
       </c>
       <c r="F19" t="n">
-        <v>0.10366761587405</v>
+        <v>0.0172655325791669</v>
       </c>
       <c r="G19" t="n">
         <v>0.011097387342098</v>
@@ -9344,7 +9344,7 @@
         <v>1</v>
       </c>
       <c r="S3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T3" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Simplifying the matrices to the raw, difference, and then only positive/net-flow for a cleaned version and for weighting based on population of origin and destination. Also re-creating the matrices accordingly.
</commit_message>
<xml_diff>
--- a/Immigration_Networks/MigrationData/Matrices/DifferenceMatrices_1990.xlsx
+++ b/Immigration_Networks/MigrationData/Matrices/DifferenceMatrices_1990.xlsx
@@ -9,10 +9,10 @@
     <sheet name="RawMatrix" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="DiffMat" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="DiffMat_Pos" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="DiffMat_PopScaled" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="DiffMat_PopScaled_Per1000" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="DiffMat_PopScaled_Pos" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="DiffMat_PopScaled_Per1000_Pos" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="DiffMat_PopScaled_dest" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="DiffMat_PopScaled_org" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="DiffMat_PopScaled_Per1000_dest" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="DiffMat_PopScaled_Per1000_org" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="DM_10000_binary" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
 </workbook>
@@ -4230,19 +4230,19 @@
         <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>-0.0176589052749834</v>
+        <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.0000402901310507417</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
         <v>0.00035495495015697</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.0142017935911534</v>
+        <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>-0.0000105733440509434</v>
+        <v>0</v>
       </c>
       <c r="H2" t="n">
         <v>0.000183329201302112</v>
@@ -4269,16 +4269,16 @@
         <v>0.0000830759945805131</v>
       </c>
       <c r="P2" t="n">
-        <v>-0.0509450890989689</v>
+        <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>-0.000421807703564121</v>
+        <v>0</v>
       </c>
       <c r="R2" t="n">
         <v>0.000331997274591508</v>
       </c>
       <c r="S2" t="n">
-        <v>-0.0392513727890685</v>
+        <v>0</v>
       </c>
       <c r="T2" t="n">
         <v>0.000379836965792243</v>
@@ -4298,13 +4298,13 @@
         <v>0.000036461596381084</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.00000791667569287645</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
         <v>0.000183818385648889</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.00000052404329115463</v>
+        <v>0</v>
       </c>
       <c r="H3" t="n">
         <v>0.0000528773343997457</v>
@@ -4316,31 +4316,31 @@
         <v>0.00000296311331352739</v>
       </c>
       <c r="K3" t="n">
-        <v>-0.00000875368277961119</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>-0.0000240940293589763</v>
+        <v>0</v>
       </c>
       <c r="M3" t="n">
-        <v>-0.0000813049706247947</v>
+        <v>0</v>
       </c>
       <c r="N3" t="n">
-        <v>-0.0000045645009631097</v>
+        <v>0</v>
       </c>
       <c r="O3" t="n">
         <v>0.0000492754673737357</v>
       </c>
       <c r="P3" t="n">
-        <v>-0.0000896729744870533</v>
+        <v>0</v>
       </c>
       <c r="Q3" t="n">
-        <v>-0.000162118424942962</v>
+        <v>0</v>
       </c>
       <c r="R3" t="n">
         <v>0.000113485643571536</v>
       </c>
       <c r="S3" t="n">
-        <v>-0.000128969667104265</v>
+        <v>0</v>
       </c>
       <c r="T3" t="n">
         <v>0.0000939212971933633</v>
@@ -4354,7 +4354,7 @@
         <v>0.000183447867407093</v>
       </c>
       <c r="C4" t="n">
-        <v>-0.000766326395012086</v>
+        <v>0</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
@@ -4363,46 +4363,46 @@
         <v>0.000217996460670207</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.00133294376735112</v>
+        <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.0000152589075953848</v>
+        <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.0000132984912861636</v>
+        <v>0</v>
       </c>
       <c r="I4" t="n">
         <v>0.0000337990343787737</v>
       </c>
       <c r="J4" t="n">
-        <v>-0.0000140747882392551</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
         <v>0.00000265934666722365</v>
       </c>
       <c r="L4" t="n">
-        <v>-0.0000202791413771384</v>
+        <v>0</v>
       </c>
       <c r="M4" t="n">
         <v>0.0000109538940139369</v>
       </c>
       <c r="N4" t="n">
-        <v>-0.0000458852465238923</v>
+        <v>0</v>
       </c>
       <c r="O4" t="n">
-        <v>-0.000138867226235073</v>
+        <v>0</v>
       </c>
       <c r="P4" t="n">
         <v>0.0221622814775544</v>
       </c>
       <c r="Q4" t="n">
-        <v>-0.000122008991145082</v>
+        <v>0</v>
       </c>
       <c r="R4" t="n">
         <v>0.000284198609196347</v>
       </c>
       <c r="S4" t="n">
-        <v>-0.00410072210180776</v>
+        <v>0</v>
       </c>
       <c r="T4" t="n">
         <v>0.000157109318162268</v>
@@ -4413,61 +4413,61 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>-0.000301136589133561</v>
+        <v>0</v>
       </c>
       <c r="C5" t="n">
         <v>0.0000310025389670208</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.0000406186743061064</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.00163315565711129</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.00021162101139862</v>
+        <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.000138367635525083</v>
+        <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>-0.000656789710428205</v>
+        <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>-0.00493302808327682</v>
+        <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>-0.0009182502429701</v>
+        <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>-0.000389118574147468</v>
+        <v>0</v>
       </c>
       <c r="M5" t="n">
-        <v>-0.000190893141748496</v>
+        <v>0</v>
       </c>
       <c r="N5" t="n">
-        <v>-0.00144478467327062</v>
+        <v>0</v>
       </c>
       <c r="O5" t="n">
-        <v>-0.000398276091665401</v>
+        <v>0</v>
       </c>
       <c r="P5" t="n">
-        <v>-0.000809027604987591</v>
+        <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>-0.000465505637101562</v>
+        <v>0</v>
       </c>
       <c r="R5" t="n">
         <v>0.00203382356276624</v>
       </c>
       <c r="S5" t="n">
-        <v>-0.00147769723055285</v>
+        <v>0</v>
       </c>
       <c r="T5" t="n">
-        <v>-0.000119388905003747</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -4478,7 +4478,7 @@
         <v>0.00582588174954741</v>
       </c>
       <c r="C6" t="n">
-        <v>-0.000348073960220642</v>
+        <v>0</v>
       </c>
       <c r="D6" t="n">
         <v>0.000120092617282382</v>
@@ -4520,13 +4520,13 @@
         <v>0.000448118518109753</v>
       </c>
       <c r="Q6" t="n">
-        <v>-0.000116876073796089</v>
+        <v>0</v>
       </c>
       <c r="R6" t="n">
         <v>0.000201162098619221</v>
       </c>
       <c r="S6" t="n">
-        <v>-0.0000744302556422625</v>
+        <v>0</v>
       </c>
       <c r="T6" t="n">
         <v>0.00100498319568252</v>
@@ -4549,7 +4549,7 @@
         <v>0.000247036266507258</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.0000226982217096807</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -4588,7 +4588,7 @@
         <v>0.00109624116128273</v>
       </c>
       <c r="S7" t="n">
-        <v>-0.000115495224272476</v>
+        <v>0</v>
       </c>
       <c r="T7" t="n">
         <v>0.0264526422238052</v>
@@ -4599,10 +4599,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>-0.0000176762048974383</v>
+        <v>0</v>
       </c>
       <c r="C8" t="n">
-        <v>-0.0000235337454886021</v>
+        <v>0</v>
       </c>
       <c r="D8" t="n">
         <v>0.000000281608504598295</v>
@@ -4611,46 +4611,46 @@
         <v>0.0000157253967172137</v>
       </c>
       <c r="F8" t="n">
-        <v>-0.000110886394581719</v>
+        <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>-0.000113470785572953</v>
+        <v>0</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>-0.0000403869817576873</v>
+        <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>-0.0101299584460397</v>
+        <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>-0.000135072649472735</v>
+        <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>-0.00040437812607482</v>
+        <v>0</v>
       </c>
       <c r="M8" t="n">
         <v>0.0000000861542225815264</v>
       </c>
       <c r="N8" t="n">
-        <v>-0.0223886369871603</v>
+        <v>0</v>
       </c>
       <c r="O8" t="n">
-        <v>-0.00194373393202347</v>
+        <v>0</v>
       </c>
       <c r="P8" t="n">
-        <v>-0.0000142885508798052</v>
+        <v>0</v>
       </c>
       <c r="Q8" t="n">
-        <v>-0.0000915748794298156</v>
+        <v>0</v>
       </c>
       <c r="R8" t="n">
         <v>0.000140501056827768</v>
       </c>
       <c r="S8" t="n">
-        <v>-0.0000808466569907334</v>
+        <v>0</v>
       </c>
       <c r="T8" t="n">
         <v>0.000031948430473861</v>
@@ -4661,22 +4661,22 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>-0.0000204543303649114</v>
+        <v>0</v>
       </c>
       <c r="C9" t="n">
-        <v>-0.000029593332650338</v>
+        <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.00000237355739589991</v>
+        <v>0</v>
       </c>
       <c r="E9" t="n">
         <v>0.000247540054960441</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.000233605632612091</v>
+        <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.000874474122557326</v>
+        <v>0</v>
       </c>
       <c r="H9" t="n">
         <v>0.000133934805096362</v>
@@ -4685,10 +4685,10 @@
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>-0.00000351869705981378</v>
+        <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>-0.00000265934666722365</v>
+        <v>0</v>
       </c>
       <c r="L9" t="n">
         <v>0.0000383496633963707</v>
@@ -4697,22 +4697,22 @@
         <v>0.000000775388003233737</v>
       </c>
       <c r="N9" t="n">
-        <v>-0.00000792781746224317</v>
+        <v>0</v>
       </c>
       <c r="O9" t="n">
         <v>0.000445108147433827</v>
       </c>
       <c r="P9" t="n">
-        <v>-0.0000199547003666245</v>
+        <v>0</v>
       </c>
       <c r="Q9" t="n">
-        <v>-0.00000358849973956122</v>
+        <v>0</v>
       </c>
       <c r="R9" t="n">
         <v>0.000541671299072233</v>
       </c>
       <c r="S9" t="n">
-        <v>-0.000102662421575535</v>
+        <v>0</v>
       </c>
       <c r="T9" t="n">
         <v>0.00111647359806515</v>
@@ -4723,10 +4723,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="n">
-        <v>-0.00000222860614423661</v>
+        <v>0</v>
       </c>
       <c r="C10" t="n">
-        <v>-0.00000225473010669242</v>
+        <v>0</v>
       </c>
       <c r="D10" t="n">
         <v>0.00000050957729403501</v>
@@ -4735,10 +4735,10 @@
         <v>0.000958529501959773</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.0000282797516382907</v>
+        <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.00000274352075957424</v>
+        <v>0</v>
       </c>
       <c r="H10" t="n">
         <v>0.0173193851157586</v>
@@ -4765,16 +4765,16 @@
         <v>0.000748905657027272</v>
       </c>
       <c r="P10" t="n">
-        <v>-0.00000886875571849978</v>
+        <v>0</v>
       </c>
       <c r="Q10" t="n">
-        <v>-0.00000817632852051925</v>
+        <v>0</v>
       </c>
       <c r="R10" t="n">
         <v>0.00183909064197061</v>
       </c>
       <c r="S10" t="n">
-        <v>-0.0000384984080908254</v>
+        <v>0</v>
       </c>
       <c r="T10" t="n">
         <v>0.0000384292531373384</v>
@@ -4785,22 +4785,22 @@
         <v>10</v>
       </c>
       <c r="B11" t="n">
-        <v>-0.00000515937586816421</v>
+        <v>0</v>
       </c>
       <c r="C11" t="n">
         <v>0.0000111327299017938</v>
       </c>
       <c r="D11" t="n">
-        <v>-0.00000016091914548474</v>
+        <v>0</v>
       </c>
       <c r="E11" t="n">
         <v>0.000298206779394851</v>
       </c>
       <c r="F11" t="n">
-        <v>-0.0000201679281420441</v>
+        <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.00000696669316476155</v>
+        <v>0</v>
       </c>
       <c r="H11" t="n">
         <v>0.000385972878043653</v>
@@ -4809,34 +4809,34 @@
         <v>0.00000229145995788297</v>
       </c>
       <c r="J11" t="n">
-        <v>-0.0423021464422454</v>
+        <v>0</v>
       </c>
       <c r="K11" t="n">
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>-0.000304789471391051</v>
+        <v>0</v>
       </c>
       <c r="M11" t="n">
         <v>0.000823892830547136</v>
       </c>
       <c r="N11" t="n">
-        <v>-0.000622694026125282</v>
+        <v>0</v>
       </c>
       <c r="O11" t="n">
         <v>0.0000545695258519056</v>
       </c>
       <c r="P11" t="n">
-        <v>-0.0000177375114369996</v>
+        <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>-0.00000499664520698398</v>
+        <v>0</v>
       </c>
       <c r="R11" t="n">
         <v>0.000884231081570292</v>
       </c>
       <c r="S11" t="n">
-        <v>-0.0000304779064052368</v>
+        <v>0</v>
       </c>
       <c r="T11" t="n">
         <v>0.0000235942450092223</v>
@@ -4847,7 +4847,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="n">
-        <v>-0.00000012211540516365</v>
+        <v>0</v>
       </c>
       <c r="C12" t="n">
         <v>0.0000169104758001931</v>
@@ -4859,19 +4859,19 @@
         <v>0.0000697387158763389</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.0000203167689401404</v>
+        <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.00000443895493683922</v>
+        <v>0</v>
       </c>
       <c r="H12" t="n">
         <v>0.000637694320246035</v>
       </c>
       <c r="I12" t="n">
-        <v>-0.0000182362021648186</v>
+        <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>-0.0183409306324062</v>
+        <v>0</v>
       </c>
       <c r="K12" t="n">
         <v>0.000168203676701896</v>
@@ -4883,22 +4883,22 @@
         <v>0.0000147077565692749</v>
       </c>
       <c r="N12" t="n">
-        <v>-0.031878714963251</v>
+        <v>0</v>
       </c>
       <c r="O12" t="n">
         <v>0.000182441399863088</v>
       </c>
       <c r="P12" t="n">
-        <v>-0.00000665156678887484</v>
+        <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>-0.00000858514494654521</v>
+        <v>0</v>
       </c>
       <c r="R12" t="n">
         <v>0.000427128198485309</v>
       </c>
       <c r="S12" t="n">
-        <v>-0.0000163618234386008</v>
+        <v>0</v>
       </c>
       <c r="T12" t="n">
         <v>0.0000183285765951469</v>
@@ -4909,58 +4909,58 @@
         <v>12</v>
       </c>
       <c r="B13" t="n">
-        <v>-0.0000613019333921523</v>
+        <v>0</v>
       </c>
       <c r="C13" t="n">
         <v>0.000930921692800633</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.00000596741831172577</v>
+        <v>0</v>
       </c>
       <c r="E13" t="n">
         <v>0.00055812563634779</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.000151594352861048</v>
+        <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.0000848333610151495</v>
+        <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>-0.0000022164152143606</v>
+        <v>0</v>
       </c>
       <c r="I13" t="n">
-        <v>-0.00000601508238944279</v>
+        <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>-0.0553081767482276</v>
+        <v>0</v>
       </c>
       <c r="K13" t="n">
-        <v>-0.00741747188544244</v>
+        <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>-0.000239936375699806</v>
+        <v>0</v>
       </c>
       <c r="M13" t="n">
         <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>-0.000521554294258482</v>
+        <v>0</v>
       </c>
       <c r="O13" t="n">
-        <v>-0.00987464076758961</v>
+        <v>0</v>
       </c>
       <c r="P13" t="n">
         <v>0.000682155127347941</v>
       </c>
       <c r="Q13" t="n">
-        <v>-0.0000931647210865832</v>
+        <v>0</v>
       </c>
       <c r="R13" t="n">
         <v>0.0164842028607365</v>
       </c>
       <c r="S13" t="n">
-        <v>-0.000126403106564877</v>
+        <v>0</v>
       </c>
       <c r="T13" t="n">
         <v>0.0000722004149853025</v>
@@ -4971,7 +4971,7 @@
         <v>13</v>
       </c>
       <c r="B14" t="n">
-        <v>-0.0000012211540516365</v>
+        <v>0</v>
       </c>
       <c r="C14" t="n">
         <v>0.00000267749200169725</v>
@@ -4983,10 +4983,10 @@
         <v>0.000216413125531632</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.0000107165374629312</v>
+        <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.00000918617063318116</v>
+        <v>0</v>
       </c>
       <c r="H14" t="n">
         <v>0.0295080856410174</v>
@@ -4995,7 +4995,7 @@
         <v>0.00000315075744208908</v>
       </c>
       <c r="J14" t="n">
-        <v>-0.0015834136769162</v>
+        <v>0</v>
       </c>
       <c r="K14" t="n">
         <v>0.000287209440060154</v>
@@ -5016,13 +5016,13 @@
         <v>0</v>
       </c>
       <c r="Q14" t="n">
-        <v>-0.0000055417337750186</v>
+        <v>0</v>
       </c>
       <c r="R14" t="n">
         <v>0.000663174316364996</v>
       </c>
       <c r="S14" t="n">
-        <v>-0.000003529020741659</v>
+        <v>0</v>
       </c>
       <c r="T14" t="n">
         <v>0.000120502796399032</v>
@@ -5033,10 +5033,10 @@
         <v>14</v>
       </c>
       <c r="B15" t="n">
-        <v>-0.00000622788566334615</v>
+        <v>0</v>
       </c>
       <c r="C15" t="n">
-        <v>-0.0000170513964318614</v>
+        <v>0</v>
       </c>
       <c r="D15" t="n">
         <v>0.00000228639285876235</v>
@@ -5045,46 +5045,46 @@
         <v>0.0000351932219437871</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.0000742715582500371</v>
+        <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>-0.00036667617342849</v>
+        <v>0</v>
       </c>
       <c r="H15" t="n">
         <v>0.00151127854544902</v>
       </c>
       <c r="I15" t="n">
-        <v>-0.00010435690558192</v>
+        <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>-0.000340572836473554</v>
+        <v>0</v>
       </c>
       <c r="K15" t="n">
-        <v>-0.0000148480188919987</v>
+        <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>-0.0000899510429401783</v>
+        <v>0</v>
       </c>
       <c r="M15" t="n">
         <v>0.000298438227022407</v>
       </c>
       <c r="N15" t="n">
-        <v>-0.000987613866281263</v>
+        <v>0</v>
       </c>
       <c r="O15" t="n">
         <v>0</v>
       </c>
       <c r="P15" t="n">
-        <v>-0.00000936146436952755</v>
+        <v>0</v>
       </c>
       <c r="Q15" t="n">
-        <v>-0.0000711794821758537</v>
+        <v>0</v>
       </c>
       <c r="R15" t="n">
         <v>0.000331386120727101</v>
       </c>
       <c r="S15" t="n">
-        <v>-0.0000471605499112612</v>
+        <v>0</v>
       </c>
       <c r="T15" t="n">
         <v>0.0000497706927984238</v>
@@ -5101,13 +5101,13 @@
         <v>0.0000512951099272525</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.000603185301956362</v>
+        <v>0</v>
       </c>
       <c r="E16" t="n">
         <v>0.000118174377160938</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.000135370705868555</v>
+        <v>0</v>
       </c>
       <c r="G16" t="n">
         <v>0</v>
@@ -5128,7 +5128,7 @@
         <v>0.00000542115660576968</v>
       </c>
       <c r="M16" t="n">
-        <v>-0.0000340801489040352</v>
+        <v>0</v>
       </c>
       <c r="N16" t="n">
         <v>0</v>
@@ -5146,7 +5146,7 @@
         <v>0.0000179928522580203</v>
       </c>
       <c r="S16" t="n">
-        <v>-0.000658322778353115</v>
+        <v>0</v>
       </c>
       <c r="T16" t="n">
         <v>0.0000181766823139717</v>
@@ -5172,7 +5172,7 @@
         <v>0.000191483686750847</v>
       </c>
       <c r="G17" t="n">
-        <v>-0.0000248458172159195</v>
+        <v>0</v>
       </c>
       <c r="H17" t="n">
         <v>0.000638327581735852</v>
@@ -5199,7 +5199,7 @@
         <v>0.000638137664253255</v>
       </c>
       <c r="P17" t="n">
-        <v>-0.0000835141163492063</v>
+        <v>0</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -5219,61 +5219,61 @@
         <v>17</v>
       </c>
       <c r="B18" t="n">
-        <v>-0.00252079777994193</v>
+        <v>0</v>
       </c>
       <c r="C18" t="n">
-        <v>-0.0039774848288371</v>
+        <v>0</v>
       </c>
       <c r="D18" t="n">
-        <v>-0.000473926998345744</v>
+        <v>0</v>
       </c>
       <c r="E18" t="n">
-        <v>-0.0182023086321776</v>
+        <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>-0.00372332698477716</v>
+        <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>-0.00840460630353796</v>
+        <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>-0.0110643447500881</v>
+        <v>0</v>
       </c>
       <c r="I18" t="n">
-        <v>-0.0128626330860848</v>
+        <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>-0.0847080018504643</v>
+        <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>-0.024368147542326</v>
+        <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>-0.0213294402736118</v>
+        <v>0</v>
       </c>
       <c r="M18" t="n">
-        <v>-0.0504591004674544</v>
+        <v>0</v>
       </c>
       <c r="N18" t="n">
-        <v>-0.0396241926238625</v>
+        <v>0</v>
       </c>
       <c r="O18" t="n">
-        <v>-0.0335639235163299</v>
+        <v>0</v>
       </c>
       <c r="P18" t="n">
-        <v>-0.00110243560667463</v>
+        <v>0</v>
       </c>
       <c r="Q18" t="n">
-        <v>-0.00627092600690691</v>
+        <v>0</v>
       </c>
       <c r="R18" t="n">
         <v>0</v>
       </c>
       <c r="S18" t="n">
-        <v>-0.00617289891729644</v>
+        <v>0</v>
       </c>
       <c r="T18" t="n">
-        <v>-0.00154324589674055</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -5326,7 +5326,7 @@
         <v>0.000505519075954488</v>
       </c>
       <c r="Q19" t="n">
-        <v>-0.00000754039185781219</v>
+        <v>0</v>
       </c>
       <c r="R19" t="n">
         <v>0.0000773632335858255</v>
@@ -5343,58 +5343,58 @@
         <v>19</v>
       </c>
       <c r="B20" t="n">
-        <v>-0.000229027442384425</v>
+        <v>0</v>
       </c>
       <c r="C20" t="n">
-        <v>-0.000261407771744652</v>
+        <v>0</v>
       </c>
       <c r="D20" t="n">
-        <v>-0.0000208055045182978</v>
+        <v>0</v>
       </c>
       <c r="E20" t="n">
         <v>0.0000848523694718303</v>
       </c>
       <c r="F20" t="n">
-        <v>-0.0014771705007064</v>
+        <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>-0.0161052375105995</v>
+        <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>-0.000199794000037362</v>
+        <v>0</v>
       </c>
       <c r="I20" t="n">
-        <v>-0.00210537431380322</v>
+        <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>-0.000140562687810456</v>
+        <v>0</v>
       </c>
       <c r="K20" t="n">
-        <v>-0.0000516356477885926</v>
+        <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>-0.000072683655232912</v>
+        <v>0</v>
       </c>
       <c r="M20" t="n">
-        <v>-0.0000175508459144652</v>
+        <v>0</v>
       </c>
       <c r="N20" t="n">
-        <v>-0.000571763804852689</v>
+        <v>0</v>
       </c>
       <c r="O20" t="n">
-        <v>-0.000400312268003159</v>
+        <v>0</v>
       </c>
       <c r="P20" t="n">
-        <v>-0.0000884412028594839</v>
+        <v>0</v>
       </c>
       <c r="Q20" t="n">
-        <v>-0.001254430491237</v>
+        <v>0</v>
       </c>
       <c r="R20" t="n">
         <v>0.000122552432809935</v>
       </c>
       <c r="S20" t="n">
-        <v>-0.00170130881754706</v>
+        <v>0</v>
       </c>
       <c r="T20" t="n">
         <v>0</v>
@@ -5481,58 +5481,58 @@
         <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>-17.6589052749834</v>
+        <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.0402901310507417</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>0.35495495015697</v>
+        <v>0.000301136589133561</v>
       </c>
       <c r="F2" t="n">
-        <v>-14.2017935911534</v>
+        <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>-0.0105733440509434</v>
+        <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>0.183329201302112</v>
+        <v>0.0000176762048974383</v>
       </c>
       <c r="I2" t="n">
-        <v>0.0639699238242328</v>
+        <v>0.0000204543303649114</v>
       </c>
       <c r="J2" t="n">
-        <v>0.0135192044929687</v>
+        <v>0.00000222860614423661</v>
       </c>
       <c r="K2" t="n">
-        <v>0.0187262327816999</v>
+        <v>0.00000515937586816421</v>
       </c>
       <c r="L2" t="n">
-        <v>0.000803134311965878</v>
+        <v>0.00000012211540516365</v>
       </c>
       <c r="M2" t="n">
-        <v>0.024713954134815</v>
+        <v>0.0000613019333921523</v>
       </c>
       <c r="N2" t="n">
-        <v>0.0096094757118099</v>
+        <v>0.0000012211540516365</v>
       </c>
       <c r="O2" t="n">
-        <v>0.0830759945805131</v>
+        <v>0.00000622788566334615</v>
       </c>
       <c r="P2" t="n">
-        <v>-50.9450890989689</v>
+        <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>-0.421807703564121</v>
+        <v>0</v>
       </c>
       <c r="R2" t="n">
-        <v>0.331997274591508</v>
+        <v>0.00252079777994193</v>
       </c>
       <c r="S2" t="n">
-        <v>-39.2513727890685</v>
+        <v>0</v>
       </c>
       <c r="T2" t="n">
-        <v>0.379836965792243</v>
+        <v>0.000229027442384425</v>
       </c>
     </row>
     <row r="3">
@@ -5540,61 +5540,61 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>3.82560088411553</v>
+        <v>0.0176589052749834</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>0.036461596381084</v>
+        <v>0.000766326395012086</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.00791667569287645</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>0.183818385648889</v>
+        <v>0.000348073960220642</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.00052404329115463</v>
+        <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>0.0528773343997457</v>
+        <v>0.0000235337454886021</v>
       </c>
       <c r="I3" t="n">
-        <v>0.020050274631476</v>
+        <v>0.000029593332650338</v>
       </c>
       <c r="J3" t="n">
-        <v>0.00296311331352739</v>
+        <v>0.00000225473010669242</v>
       </c>
       <c r="K3" t="n">
-        <v>-0.00875368277961119</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>-0.0240940293589763</v>
+        <v>0</v>
       </c>
       <c r="M3" t="n">
-        <v>-0.0813049706247947</v>
+        <v>0</v>
       </c>
       <c r="N3" t="n">
-        <v>-0.0045645009631097</v>
+        <v>0</v>
       </c>
       <c r="O3" t="n">
-        <v>0.0492754673737357</v>
+        <v>0.0000170513964318614</v>
       </c>
       <c r="P3" t="n">
-        <v>-0.0896729744870533</v>
+        <v>0</v>
       </c>
       <c r="Q3" t="n">
-        <v>-0.162118424942962</v>
+        <v>0</v>
       </c>
       <c r="R3" t="n">
-        <v>0.113485643571536</v>
+        <v>0.0039774848288371</v>
       </c>
       <c r="S3" t="n">
-        <v>-0.128969667104265</v>
+        <v>0</v>
       </c>
       <c r="T3" t="n">
-        <v>0.0939212971933633</v>
+        <v>0.000261407771744652</v>
       </c>
     </row>
     <row r="4">
@@ -5602,61 +5602,61 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>0.183447867407093</v>
+        <v>0.0000402901310507417</v>
       </c>
       <c r="C4" t="n">
-        <v>-0.766326395012086</v>
+        <v>0</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>0.217996460670207</v>
+        <v>0.0000406186743061064</v>
       </c>
       <c r="F4" t="n">
-        <v>-1.33294376735112</v>
+        <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.0152589075953848</v>
+        <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.0132984912861636</v>
+        <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>0.0337990343787737</v>
+        <v>0.00000237355739589991</v>
       </c>
       <c r="J4" t="n">
-        <v>-0.0140747882392551</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>0.00265934666722365</v>
+        <v>0.00000016091914548474</v>
       </c>
       <c r="L4" t="n">
-        <v>-0.0202791413771384</v>
+        <v>0</v>
       </c>
       <c r="M4" t="n">
-        <v>0.0109538940139369</v>
+        <v>0.00000596741831172577</v>
       </c>
       <c r="N4" t="n">
-        <v>-0.0458852465238923</v>
+        <v>0</v>
       </c>
       <c r="O4" t="n">
-        <v>-0.138867226235073</v>
+        <v>0</v>
       </c>
       <c r="P4" t="n">
-        <v>22.1622814775544</v>
+        <v>0.000603185301956362</v>
       </c>
       <c r="Q4" t="n">
-        <v>-0.122008991145082</v>
+        <v>0</v>
       </c>
       <c r="R4" t="n">
-        <v>0.284198609196347</v>
+        <v>0.000473926998345744</v>
       </c>
       <c r="S4" t="n">
-        <v>-4.10072210180776</v>
+        <v>0</v>
       </c>
       <c r="T4" t="n">
-        <v>0.157109318162268</v>
+        <v>0.0000208055045182978</v>
       </c>
     </row>
     <row r="5">
@@ -5664,61 +5664,61 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>-0.301136589133561</v>
+        <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0310025389670208</v>
+        <v>0.00000791667569287645</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.0406186743061064</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>-1.63315565711129</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.21162101139862</v>
+        <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.138367635525083</v>
+        <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>-0.656789710428205</v>
+        <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>-4.93302808327682</v>
+        <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>-0.9182502429701</v>
+        <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>-0.389118574147468</v>
+        <v>0</v>
       </c>
       <c r="M5" t="n">
-        <v>-0.190893141748496</v>
+        <v>0</v>
       </c>
       <c r="N5" t="n">
-        <v>-1.44478467327062</v>
+        <v>0</v>
       </c>
       <c r="O5" t="n">
-        <v>-0.398276091665401</v>
+        <v>0</v>
       </c>
       <c r="P5" t="n">
-        <v>-0.809027604987591</v>
+        <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>-0.465505637101562</v>
+        <v>0</v>
       </c>
       <c r="R5" t="n">
-        <v>2.03382356276624</v>
+        <v>0.0182023086321776</v>
       </c>
       <c r="S5" t="n">
-        <v>-1.47769723055285</v>
+        <v>0</v>
       </c>
       <c r="T5" t="n">
-        <v>-0.119388905003747</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -5726,61 +5726,61 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>5.82588174954741</v>
+        <v>0.0142017935911534</v>
       </c>
       <c r="C6" t="n">
-        <v>-0.348073960220642</v>
+        <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>0.120092617282382</v>
+        <v>0.00133294376735112</v>
       </c>
       <c r="E6" t="n">
-        <v>0.789688400364426</v>
+        <v>0.00163315565711129</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>0.00940195316483307</v>
+        <v>0.0000226982217096807</v>
       </c>
       <c r="H6" t="n">
-        <v>0.471779809913899</v>
+        <v>0.000110886394581719</v>
       </c>
       <c r="I6" t="n">
-        <v>0.299703866991443</v>
+        <v>0.000233605632612091</v>
       </c>
       <c r="J6" t="n">
-        <v>0.0703739411962755</v>
+        <v>0.0000282797516382907</v>
       </c>
       <c r="K6" t="n">
-        <v>0.0300284561174004</v>
+        <v>0.0000201679281420441</v>
       </c>
       <c r="L6" t="n">
-        <v>0.0548139167916712</v>
+        <v>0.0000203167689401404</v>
       </c>
       <c r="M6" t="n">
-        <v>0.0250708787712242</v>
+        <v>0.000151594352861048</v>
       </c>
       <c r="N6" t="n">
-        <v>0.0345941125625156</v>
+        <v>0.0000107165374629312</v>
       </c>
       <c r="O6" t="n">
-        <v>0.406420797016432</v>
+        <v>0.0000742715582500371</v>
       </c>
       <c r="P6" t="n">
-        <v>0.448118518109753</v>
+        <v>0.000135370705868555</v>
       </c>
       <c r="Q6" t="n">
-        <v>-0.116876073796089</v>
+        <v>0</v>
       </c>
       <c r="R6" t="n">
-        <v>0.201162098619221</v>
+        <v>0.00372332698477716</v>
       </c>
       <c r="S6" t="n">
-        <v>-0.0744302556422625</v>
+        <v>0</v>
       </c>
       <c r="T6" t="n">
-        <v>1.00498319568252</v>
+        <v>0.0014771705007064</v>
       </c>
     </row>
     <row r="7">
@@ -5788,61 +5788,61 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>0.010471395992783</v>
+        <v>0.0000105733440509434</v>
       </c>
       <c r="C7" t="n">
-        <v>0.0023956507383607</v>
+        <v>0.00000052404329115463</v>
       </c>
       <c r="D7" t="n">
-        <v>0.00331895737562276</v>
+        <v>0.0000152589075953848</v>
       </c>
       <c r="E7" t="n">
-        <v>0.247036266507258</v>
+        <v>0.00021162101139862</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.0226982217096807</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>1.16551777200877</v>
+        <v>0.000113470785572953</v>
       </c>
       <c r="I7" t="n">
-        <v>2.70850567021767</v>
+        <v>0.000874474122557326</v>
       </c>
       <c r="J7" t="n">
-        <v>0.0164823178064961</v>
+        <v>0.00000274352075957424</v>
       </c>
       <c r="K7" t="n">
-        <v>0.0250421811163561</v>
+        <v>0.00000696669316476155</v>
       </c>
       <c r="L7" t="n">
-        <v>0.0289128352307716</v>
+        <v>0.00000443895493683922</v>
       </c>
       <c r="M7" t="n">
-        <v>0.0338709172206229</v>
+        <v>0.0000848333610151495</v>
       </c>
       <c r="N7" t="n">
-        <v>0.0715905940529838</v>
+        <v>0.00000918617063318116</v>
       </c>
       <c r="O7" t="n">
-        <v>4.8440635075255</v>
+        <v>0.00036667617342849</v>
       </c>
       <c r="P7" t="n">
         <v>0</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.0366117821529917</v>
+        <v>0.0000248458172159195</v>
       </c>
       <c r="R7" t="n">
-        <v>1.09624116128273</v>
+        <v>0.00840460630353796</v>
       </c>
       <c r="S7" t="n">
-        <v>-0.115495224272476</v>
+        <v>0</v>
       </c>
       <c r="T7" t="n">
-        <v>26.4526422238052</v>
+        <v>0.0161052375105995</v>
       </c>
     </row>
     <row r="8">
@@ -5850,61 +5850,61 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>-0.0176762048974383</v>
+        <v>0</v>
       </c>
       <c r="C8" t="n">
-        <v>-0.0235337454886021</v>
+        <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>0.000281608504598295</v>
+        <v>0.0000132984912861636</v>
       </c>
       <c r="E8" t="n">
-        <v>0.0157253967172137</v>
+        <v>0.000138367635525083</v>
       </c>
       <c r="F8" t="n">
-        <v>-0.110886394581719</v>
+        <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>-0.113470785572953</v>
+        <v>0</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>-0.0403869817576873</v>
+        <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>-10.1299584460397</v>
+        <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>-0.135072649472735</v>
+        <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>-0.40437812607482</v>
+        <v>0</v>
       </c>
       <c r="M8" t="n">
-        <v>0.0000861542225815264</v>
+        <v>0.0000022164152143606</v>
       </c>
       <c r="N8" t="n">
-        <v>-22.3886369871603</v>
+        <v>0</v>
       </c>
       <c r="O8" t="n">
-        <v>-1.94373393202347</v>
+        <v>0</v>
       </c>
       <c r="P8" t="n">
-        <v>-0.0142885508798052</v>
+        <v>0</v>
       </c>
       <c r="Q8" t="n">
-        <v>-0.0915748794298156</v>
+        <v>0</v>
       </c>
       <c r="R8" t="n">
-        <v>0.140501056827768</v>
+        <v>0.0110643447500881</v>
       </c>
       <c r="S8" t="n">
-        <v>-0.0808466569907334</v>
+        <v>0</v>
       </c>
       <c r="T8" t="n">
-        <v>0.031948430473861</v>
+        <v>0.000199794000037362</v>
       </c>
     </row>
     <row r="9">
@@ -5912,61 +5912,61 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>-0.0204543303649114</v>
+        <v>0</v>
       </c>
       <c r="C9" t="n">
-        <v>-0.029593332650338</v>
+        <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.00237355739589991</v>
+        <v>0</v>
       </c>
       <c r="E9" t="n">
-        <v>0.247540054960441</v>
+        <v>0.000656789710428205</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.233605632612091</v>
+        <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.874474122557326</v>
+        <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>0.133934805096362</v>
+        <v>0.0000403869817576873</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>-0.00351869705981378</v>
+        <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>-0.00265934666722365</v>
+        <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>0.0383496633963707</v>
+        <v>0.0000182362021648186</v>
       </c>
       <c r="M9" t="n">
-        <v>0.000775388003233737</v>
+        <v>0.00000601508238944279</v>
       </c>
       <c r="N9" t="n">
-        <v>-0.00792781746224317</v>
+        <v>0</v>
       </c>
       <c r="O9" t="n">
-        <v>0.445108147433827</v>
+        <v>0.00010435690558192</v>
       </c>
       <c r="P9" t="n">
-        <v>-0.0199547003666245</v>
+        <v>0</v>
       </c>
       <c r="Q9" t="n">
-        <v>-0.00358849973956122</v>
+        <v>0</v>
       </c>
       <c r="R9" t="n">
-        <v>0.541671299072233</v>
+        <v>0.0128626330860848</v>
       </c>
       <c r="S9" t="n">
-        <v>-0.102662421575535</v>
+        <v>0</v>
       </c>
       <c r="T9" t="n">
-        <v>1.11647359806515</v>
+        <v>0.00210537431380322</v>
       </c>
     </row>
     <row r="10">
@@ -5974,61 +5974,61 @@
         <v>9</v>
       </c>
       <c r="B10" t="n">
-        <v>-0.00222860614423661</v>
+        <v>0</v>
       </c>
       <c r="C10" t="n">
-        <v>-0.00225473010669242</v>
+        <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>0.00050957729403501</v>
+        <v>0.0000140747882392551</v>
       </c>
       <c r="E10" t="n">
-        <v>0.958529501959773</v>
+        <v>0.00493302808327682</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.0282797516382907</v>
+        <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.00274352075957424</v>
+        <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>17.3193851157586</v>
+        <v>0.0101299584460397</v>
       </c>
       <c r="I10" t="n">
-        <v>0.00181407246665735</v>
+        <v>0.00000351869705981378</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>25.3103319053011</v>
+        <v>0.0423021464422454</v>
       </c>
       <c r="L10" t="n">
-        <v>19.8848024299632</v>
+        <v>0.0183409306324062</v>
       </c>
       <c r="M10" t="n">
-        <v>3.67569605996432</v>
+        <v>0.0553081767482276</v>
       </c>
       <c r="N10" t="n">
-        <v>2.05402543339937</v>
+        <v>0.0015834136769162</v>
       </c>
       <c r="O10" t="n">
-        <v>0.748905657027272</v>
+        <v>0.000340572836473554</v>
       </c>
       <c r="P10" t="n">
-        <v>-0.00886875571849978</v>
+        <v>0</v>
       </c>
       <c r="Q10" t="n">
-        <v>-0.00817632852051925</v>
+        <v>0</v>
       </c>
       <c r="R10" t="n">
-        <v>1.83909064197061</v>
+        <v>0.0847080018504643</v>
       </c>
       <c r="S10" t="n">
-        <v>-0.0384984080908254</v>
+        <v>0</v>
       </c>
       <c r="T10" t="n">
-        <v>0.0384292531373384</v>
+        <v>0.000140562687810456</v>
       </c>
     </row>
     <row r="11">
@@ -6036,61 +6036,61 @@
         <v>10</v>
       </c>
       <c r="B11" t="n">
-        <v>-0.00515937586816421</v>
+        <v>0</v>
       </c>
       <c r="C11" t="n">
-        <v>0.0111327299017938</v>
+        <v>0.00000875368277961119</v>
       </c>
       <c r="D11" t="n">
-        <v>-0.00016091914548474</v>
+        <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>0.298206779394851</v>
+        <v>0.0009182502429701</v>
       </c>
       <c r="F11" t="n">
-        <v>-0.0201679281420441</v>
+        <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.00696669316476155</v>
+        <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>0.385972878043653</v>
+        <v>0.000135072649472735</v>
       </c>
       <c r="I11" t="n">
-        <v>0.00229145995788297</v>
+        <v>0.00000265934666722365</v>
       </c>
       <c r="J11" t="n">
-        <v>-42.3021464422454</v>
+        <v>0</v>
       </c>
       <c r="K11" t="n">
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>-0.304789471391051</v>
+        <v>0</v>
       </c>
       <c r="M11" t="n">
-        <v>0.823892830547136</v>
+        <v>0.00741747188544244</v>
       </c>
       <c r="N11" t="n">
-        <v>-0.622694026125282</v>
+        <v>0</v>
       </c>
       <c r="O11" t="n">
-        <v>0.0545695258519056</v>
+        <v>0.0000148480188919987</v>
       </c>
       <c r="P11" t="n">
-        <v>-0.0177375114369996</v>
+        <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>-0.00499664520698398</v>
+        <v>0</v>
       </c>
       <c r="R11" t="n">
-        <v>0.884231081570292</v>
+        <v>0.024368147542326</v>
       </c>
       <c r="S11" t="n">
-        <v>-0.0304779064052368</v>
+        <v>0</v>
       </c>
       <c r="T11" t="n">
-        <v>0.0235942450092223</v>
+        <v>0.0000516356477885926</v>
       </c>
     </row>
     <row r="12">
@@ -6098,61 +6098,61 @@
         <v>11</v>
       </c>
       <c r="B12" t="n">
-        <v>-0.00012211540516365</v>
+        <v>0</v>
       </c>
       <c r="C12" t="n">
-        <v>0.0169104758001931</v>
+        <v>0.0000240940293589763</v>
       </c>
       <c r="D12" t="n">
-        <v>0.000677201403914947</v>
+        <v>0.0000202791413771384</v>
       </c>
       <c r="E12" t="n">
-        <v>0.0697387158763389</v>
+        <v>0.000389118574147468</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.0203167689401404</v>
+        <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.00443895493683922</v>
+        <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>0.637694320246035</v>
+        <v>0.00040437812607482</v>
       </c>
       <c r="I12" t="n">
-        <v>-0.0182362021648186</v>
+        <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>-18.3409306324062</v>
+        <v>0</v>
       </c>
       <c r="K12" t="n">
-        <v>0.168203676701896</v>
+        <v>0.000304789471391051</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
       </c>
       <c r="M12" t="n">
-        <v>0.0147077565692749</v>
+        <v>0.000239936375699806</v>
       </c>
       <c r="N12" t="n">
-        <v>-31.878714963251</v>
+        <v>0</v>
       </c>
       <c r="O12" t="n">
-        <v>0.182441399863087</v>
+        <v>0.0000899510429401783</v>
       </c>
       <c r="P12" t="n">
-        <v>-0.00665156678887484</v>
+        <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>-0.00858514494654521</v>
+        <v>0</v>
       </c>
       <c r="R12" t="n">
-        <v>0.427128198485309</v>
+        <v>0.0213294402736118</v>
       </c>
       <c r="S12" t="n">
-        <v>-0.0163618234386008</v>
+        <v>0</v>
       </c>
       <c r="T12" t="n">
-        <v>0.0183285765951469</v>
+        <v>0.000072683655232912</v>
       </c>
     </row>
     <row r="13">
@@ -6160,61 +6160,61 @@
         <v>12</v>
       </c>
       <c r="B13" t="n">
-        <v>-0.0613019333921523</v>
+        <v>0</v>
       </c>
       <c r="C13" t="n">
-        <v>0.930921692800633</v>
+        <v>0.0000813049706247947</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.00596741831172577</v>
+        <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>0.55812563634779</v>
+        <v>0.000190893141748496</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.151594352861048</v>
+        <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.0848333610151495</v>
+        <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>-0.0022164152143606</v>
+        <v>0</v>
       </c>
       <c r="I13" t="n">
-        <v>-0.00601508238944279</v>
+        <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>-55.3081767482276</v>
+        <v>0</v>
       </c>
       <c r="K13" t="n">
-        <v>-7.41747188544244</v>
+        <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>-0.239936375699806</v>
+        <v>0</v>
       </c>
       <c r="M13" t="n">
         <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>-0.521554294258482</v>
+        <v>0</v>
       </c>
       <c r="O13" t="n">
-        <v>-9.87464076758961</v>
+        <v>0</v>
       </c>
       <c r="P13" t="n">
-        <v>0.682155127347941</v>
+        <v>0.0000340801489040352</v>
       </c>
       <c r="Q13" t="n">
-        <v>-0.0931647210865832</v>
+        <v>0</v>
       </c>
       <c r="R13" t="n">
-        <v>16.4842028607365</v>
+        <v>0.0504591004674544</v>
       </c>
       <c r="S13" t="n">
-        <v>-0.126403106564877</v>
+        <v>0</v>
       </c>
       <c r="T13" t="n">
-        <v>0.0722004149853025</v>
+        <v>0.0000175508459144652</v>
       </c>
     </row>
     <row r="14">
@@ -6222,61 +6222,61 @@
         <v>13</v>
       </c>
       <c r="B14" t="n">
-        <v>-0.0012211540516365</v>
+        <v>0</v>
       </c>
       <c r="C14" t="n">
-        <v>0.00267749200169725</v>
+        <v>0.0000045645009631097</v>
       </c>
       <c r="D14" t="n">
-        <v>0.00128064819948272</v>
+        <v>0.0000458852465238923</v>
       </c>
       <c r="E14" t="n">
-        <v>0.216413125531632</v>
+        <v>0.00144478467327062</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.0107165374629312</v>
+        <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.00918617063318116</v>
+        <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>29.5080856410174</v>
+        <v>0.0223886369871603</v>
       </c>
       <c r="I14" t="n">
-        <v>0.00315075744208908</v>
+        <v>0.00000792781746224317</v>
       </c>
       <c r="J14" t="n">
-        <v>-1.5834136769162</v>
+        <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>0.287209440060154</v>
+        <v>0.000622694026125282</v>
       </c>
       <c r="L14" t="n">
-        <v>26.643378448734</v>
+        <v>0.031878714963251</v>
       </c>
       <c r="M14" t="n">
-        <v>0.0267201167463562</v>
+        <v>0.000521554294258482</v>
       </c>
       <c r="N14" t="n">
         <v>0</v>
       </c>
       <c r="O14" t="n">
-        <v>1.67414418490436</v>
+        <v>0.000987613866281263</v>
       </c>
       <c r="P14" t="n">
         <v>0</v>
       </c>
       <c r="Q14" t="n">
-        <v>-0.0055417337750186</v>
+        <v>0</v>
       </c>
       <c r="R14" t="n">
-        <v>0.663174316364996</v>
+        <v>0.0396241926238625</v>
       </c>
       <c r="S14" t="n">
-        <v>-0.003529020741659</v>
+        <v>0</v>
       </c>
       <c r="T14" t="n">
-        <v>0.120502796399032</v>
+        <v>0.000571763804852689</v>
       </c>
     </row>
     <row r="15">
@@ -6284,61 +6284,61 @@
         <v>14</v>
       </c>
       <c r="B15" t="n">
-        <v>-0.00622788566334615</v>
+        <v>0</v>
       </c>
       <c r="C15" t="n">
-        <v>-0.0170513964318614</v>
+        <v>0</v>
       </c>
       <c r="D15" t="n">
-        <v>0.00228639285876235</v>
+        <v>0.000138867226235073</v>
       </c>
       <c r="E15" t="n">
-        <v>0.0351932219437871</v>
+        <v>0.000398276091665401</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.0742715582500371</v>
+        <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>-0.36667617342849</v>
+        <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>1.51127854544902</v>
+        <v>0.00194373393202347</v>
       </c>
       <c r="I15" t="n">
-        <v>-0.10435690558192</v>
+        <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>-0.340572836473554</v>
+        <v>0</v>
       </c>
       <c r="K15" t="n">
-        <v>-0.0148480188919987</v>
+        <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>-0.0899510429401783</v>
+        <v>0</v>
       </c>
       <c r="M15" t="n">
-        <v>0.298438227022407</v>
+        <v>0.00987464076758961</v>
       </c>
       <c r="N15" t="n">
-        <v>-0.987613866281263</v>
+        <v>0</v>
       </c>
       <c r="O15" t="n">
         <v>0</v>
       </c>
       <c r="P15" t="n">
-        <v>-0.00936146436952755</v>
+        <v>0</v>
       </c>
       <c r="Q15" t="n">
-        <v>-0.0711794821758537</v>
+        <v>0</v>
       </c>
       <c r="R15" t="n">
-        <v>0.331386120727101</v>
+        <v>0.0335639235163299</v>
       </c>
       <c r="S15" t="n">
-        <v>-0.0471605499112612</v>
+        <v>0</v>
       </c>
       <c r="T15" t="n">
-        <v>0.0497706927984238</v>
+        <v>0.000400312268003159</v>
       </c>
     </row>
     <row r="16">
@@ -6346,61 +6346,61 @@
         <v>15</v>
       </c>
       <c r="B16" t="n">
-        <v>6.31324433155554</v>
+        <v>0.0509450890989689</v>
       </c>
       <c r="C16" t="n">
-        <v>0.0512951099272525</v>
+        <v>0.0000896729744870533</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.603185301956362</v>
+        <v>0</v>
       </c>
       <c r="E16" t="n">
-        <v>0.118174377160938</v>
+        <v>0.000809027604987591</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.135370705868555</v>
+        <v>0</v>
       </c>
       <c r="G16" t="n">
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>0.0183645832047021</v>
+        <v>0.0000142885508798052</v>
       </c>
       <c r="I16" t="n">
-        <v>0.00773367735785501</v>
+        <v>0.0000199547003666245</v>
       </c>
       <c r="J16" t="n">
-        <v>0.00666700495543663</v>
+        <v>0.00000886875571849978</v>
       </c>
       <c r="K16" t="n">
-        <v>0.00797804000167096</v>
+        <v>0.0000177375114369996</v>
       </c>
       <c r="L16" t="n">
-        <v>0.00542115660576968</v>
+        <v>0.00000665156678887484</v>
       </c>
       <c r="M16" t="n">
-        <v>-0.0340801489040352</v>
+        <v>0</v>
       </c>
       <c r="N16" t="n">
         <v>0</v>
       </c>
       <c r="O16" t="n">
-        <v>0.0154749401669583</v>
+        <v>0.00000936146436952755</v>
       </c>
       <c r="P16" t="n">
         <v>0</v>
       </c>
       <c r="Q16" t="n">
-        <v>0.0153987520469779</v>
+        <v>0.0000835141163492063</v>
       </c>
       <c r="R16" t="n">
-        <v>0.0179928522580203</v>
+        <v>0.00110243560667463</v>
       </c>
       <c r="S16" t="n">
-        <v>-0.658322778353115</v>
+        <v>0</v>
       </c>
       <c r="T16" t="n">
-        <v>0.0181766823139717</v>
+        <v>0.0000884412028594839</v>
       </c>
     </row>
     <row r="17">
@@ -6408,61 +6408,61 @@
         <v>16</v>
       </c>
       <c r="B17" t="n">
-        <v>0.283490913087413</v>
+        <v>0.000421807703564121</v>
       </c>
       <c r="C17" t="n">
-        <v>0.502945734424078</v>
+        <v>0.000162118424942962</v>
       </c>
       <c r="D17" t="n">
-        <v>0.0180095343655005</v>
+        <v>0.000122008991145082</v>
       </c>
       <c r="E17" t="n">
-        <v>0.36877314772999</v>
+        <v>0.000465505637101562</v>
       </c>
       <c r="F17" t="n">
-        <v>0.191483686750847</v>
+        <v>0.000116876073796089</v>
       </c>
       <c r="G17" t="n">
-        <v>-0.0248458172159195</v>
+        <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>0.638327581735852</v>
+        <v>0.0000915748794298156</v>
       </c>
       <c r="I17" t="n">
-        <v>0.00754272236136476</v>
+        <v>0.00000358849973956122</v>
       </c>
       <c r="J17" t="n">
-        <v>0.0333350247771831</v>
+        <v>0.00000817632852051925</v>
       </c>
       <c r="K17" t="n">
-        <v>0.0121886722247751</v>
+        <v>0.00000499664520698398</v>
       </c>
       <c r="L17" t="n">
-        <v>0.0379480962403877</v>
+        <v>0.00000858514494654521</v>
       </c>
       <c r="M17" t="n">
-        <v>0.0252431872163872</v>
+        <v>0.0000931647210865832</v>
       </c>
       <c r="N17" t="n">
-        <v>0.0293089009210202</v>
+        <v>0.0000055417337750186</v>
       </c>
       <c r="O17" t="n">
-        <v>0.638137664253255</v>
+        <v>0.0000711794821758537</v>
       </c>
       <c r="P17" t="n">
-        <v>-0.0835141163492063</v>
+        <v>0</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
       </c>
       <c r="R17" t="n">
-        <v>0.555076476598096</v>
+        <v>0.00627092600690691</v>
       </c>
       <c r="S17" t="n">
-        <v>0.0532561311923085</v>
+        <v>0.00000754039185781219</v>
       </c>
       <c r="T17" t="n">
-        <v>1.39823748964524</v>
+        <v>0.001254430491237</v>
       </c>
     </row>
     <row r="18">
@@ -6470,61 +6470,61 @@
         <v>17</v>
       </c>
       <c r="B18" t="n">
-        <v>-2.52079777994193</v>
+        <v>0</v>
       </c>
       <c r="C18" t="n">
-        <v>-3.9774848288371</v>
+        <v>0</v>
       </c>
       <c r="D18" t="n">
-        <v>-0.473926998345744</v>
+        <v>0</v>
       </c>
       <c r="E18" t="n">
-        <v>-18.2023086321776</v>
+        <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>-3.72332698477716</v>
+        <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>-8.40460630353796</v>
+        <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>-11.0643447500881</v>
+        <v>0</v>
       </c>
       <c r="I18" t="n">
-        <v>-12.8626330860848</v>
+        <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>-84.7080018504643</v>
+        <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>-24.368147542326</v>
+        <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>-21.3294402736118</v>
+        <v>0</v>
       </c>
       <c r="M18" t="n">
-        <v>-50.4591004674544</v>
+        <v>0</v>
       </c>
       <c r="N18" t="n">
-        <v>-39.6241926238625</v>
+        <v>0</v>
       </c>
       <c r="O18" t="n">
-        <v>-33.5639235163299</v>
+        <v>0</v>
       </c>
       <c r="P18" t="n">
-        <v>-1.10243560667463</v>
+        <v>0</v>
       </c>
       <c r="Q18" t="n">
-        <v>-6.27092600690691</v>
+        <v>0</v>
       </c>
       <c r="R18" t="n">
         <v>0</v>
       </c>
       <c r="S18" t="n">
-        <v>-6.17289891729644</v>
+        <v>0</v>
       </c>
       <c r="T18" t="n">
-        <v>-1.54324589674055</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -6532,61 +6532,61 @@
         <v>18</v>
       </c>
       <c r="B19" t="n">
-        <v>3.73511336888927</v>
+        <v>0.0392513727890685</v>
       </c>
       <c r="C19" t="n">
-        <v>0.056650093930647</v>
+        <v>0.000128969667104265</v>
       </c>
       <c r="D19" t="n">
-        <v>0.0857028548994144</v>
+        <v>0.00410072210180776</v>
       </c>
       <c r="E19" t="n">
-        <v>0.165746401097222</v>
+        <v>0.00147769723055285</v>
       </c>
       <c r="F19" t="n">
-        <v>0.0172655325791669</v>
+        <v>0.0000744302556422625</v>
       </c>
       <c r="G19" t="n">
-        <v>0.011097387342098</v>
+        <v>0.000115495224272476</v>
       </c>
       <c r="H19" t="n">
-        <v>0.0797909477169815</v>
+        <v>0.0000808466569907334</v>
       </c>
       <c r="I19" t="n">
-        <v>0.0305527994384395</v>
+        <v>0.000102662421575535</v>
       </c>
       <c r="J19" t="n">
-        <v>0.0222233498514554</v>
+        <v>0.0000384984080908254</v>
       </c>
       <c r="K19" t="n">
-        <v>0.0105265805577603</v>
+        <v>0.0000304779064052368</v>
       </c>
       <c r="L19" t="n">
-        <v>0.0102399624775649</v>
+        <v>0.0000163618234386008</v>
       </c>
       <c r="M19" t="n">
-        <v>0.00484925195673163</v>
+        <v>0.000126403106564877</v>
       </c>
       <c r="N19" t="n">
-        <v>0.00264260582074772</v>
+        <v>0.000003529020741659</v>
       </c>
       <c r="O19" t="n">
-        <v>0.0598635843300756</v>
+        <v>0.0000471605499112612</v>
       </c>
       <c r="P19" t="n">
-        <v>0.505519075954488</v>
+        <v>0.000658322778353115</v>
       </c>
       <c r="Q19" t="n">
-        <v>-0.00754039185781219</v>
+        <v>0</v>
       </c>
       <c r="R19" t="n">
-        <v>0.0773632335858255</v>
+        <v>0.00617289891729644</v>
       </c>
       <c r="S19" t="n">
         <v>0</v>
       </c>
       <c r="T19" t="n">
-        <v>0.268498457690785</v>
+        <v>0.00170130881754706</v>
       </c>
     </row>
     <row r="20">
@@ -6594,58 +6594,58 @@
         <v>19</v>
       </c>
       <c r="B20" t="n">
-        <v>-0.229027442384425</v>
+        <v>0</v>
       </c>
       <c r="C20" t="n">
-        <v>-0.261407771744652</v>
+        <v>0</v>
       </c>
       <c r="D20" t="n">
-        <v>-0.0208055045182978</v>
+        <v>0</v>
       </c>
       <c r="E20" t="n">
-        <v>0.0848523694718303</v>
+        <v>0.000119388905003747</v>
       </c>
       <c r="F20" t="n">
-        <v>-1.4771705007064</v>
+        <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>-16.1052375105995</v>
+        <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>-0.199794000037362</v>
+        <v>0</v>
       </c>
       <c r="I20" t="n">
-        <v>-2.10537431380322</v>
+        <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>-0.140562687810456</v>
+        <v>0</v>
       </c>
       <c r="K20" t="n">
-        <v>-0.0516356477885926</v>
+        <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>-0.072683655232912</v>
+        <v>0</v>
       </c>
       <c r="M20" t="n">
-        <v>-0.0175508459144652</v>
+        <v>0</v>
       </c>
       <c r="N20" t="n">
-        <v>-0.571763804852689</v>
+        <v>0</v>
       </c>
       <c r="O20" t="n">
-        <v>-0.400312268003159</v>
+        <v>0</v>
       </c>
       <c r="P20" t="n">
-        <v>-0.0884412028594839</v>
+        <v>0</v>
       </c>
       <c r="Q20" t="n">
-        <v>-1.254430491237</v>
+        <v>0</v>
       </c>
       <c r="R20" t="n">
-        <v>0.122552432809935</v>
+        <v>0.00154324589674055</v>
       </c>
       <c r="S20" t="n">
-        <v>-1.70130881754706</v>
+        <v>0</v>
       </c>
       <c r="T20" t="n">
         <v>0</v>
@@ -6738,7 +6738,7 @@
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>0.00035495495015697</v>
+        <v>0.35495495015697</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
@@ -6747,28 +6747,28 @@
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>0.000183329201302112</v>
+        <v>0.183329201302112</v>
       </c>
       <c r="I2" t="n">
-        <v>0.0000639699238242328</v>
+        <v>0.0639699238242328</v>
       </c>
       <c r="J2" t="n">
-        <v>0.0000135192044929687</v>
+        <v>0.0135192044929687</v>
       </c>
       <c r="K2" t="n">
-        <v>0.0000187262327816999</v>
+        <v>0.0187262327816999</v>
       </c>
       <c r="L2" t="n">
-        <v>0.000000803134311965878</v>
+        <v>0.000803134311965878</v>
       </c>
       <c r="M2" t="n">
-        <v>0.000024713954134815</v>
+        <v>0.024713954134815</v>
       </c>
       <c r="N2" t="n">
-        <v>0.0000096094757118099</v>
+        <v>0.0096094757118099</v>
       </c>
       <c r="O2" t="n">
-        <v>0.0000830759945805131</v>
+        <v>0.0830759945805131</v>
       </c>
       <c r="P2" t="n">
         <v>0</v>
@@ -6777,13 +6777,13 @@
         <v>0</v>
       </c>
       <c r="R2" t="n">
-        <v>0.000331997274591508</v>
+        <v>0.331997274591508</v>
       </c>
       <c r="S2" t="n">
         <v>0</v>
       </c>
       <c r="T2" t="n">
-        <v>0.000379836965792243</v>
+        <v>0.379836965792243</v>
       </c>
     </row>
     <row r="3">
@@ -6791,31 +6791,31 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>0.00382560088411553</v>
+        <v>3.82560088411553</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>0.000036461596381084</v>
+        <v>0.036461596381084</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>0.000183818385648889</v>
+        <v>0.183818385648889</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>0.0000528773343997457</v>
+        <v>0.0528773343997457</v>
       </c>
       <c r="I3" t="n">
-        <v>0.000020050274631476</v>
+        <v>0.020050274631476</v>
       </c>
       <c r="J3" t="n">
-        <v>0.00000296311331352739</v>
+        <v>0.00296311331352739</v>
       </c>
       <c r="K3" t="n">
         <v>0</v>
@@ -6830,7 +6830,7 @@
         <v>0</v>
       </c>
       <c r="O3" t="n">
-        <v>0.0000492754673737357</v>
+        <v>0.0492754673737357</v>
       </c>
       <c r="P3" t="n">
         <v>0</v>
@@ -6839,13 +6839,13 @@
         <v>0</v>
       </c>
       <c r="R3" t="n">
-        <v>0.000113485643571536</v>
+        <v>0.113485643571536</v>
       </c>
       <c r="S3" t="n">
         <v>0</v>
       </c>
       <c r="T3" t="n">
-        <v>0.0000939212971933633</v>
+        <v>0.0939212971933633</v>
       </c>
     </row>
     <row r="4">
@@ -6853,7 +6853,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>0.000183447867407093</v>
+        <v>0.183447867407093</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
@@ -6862,7 +6862,7 @@
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>0.000217996460670207</v>
+        <v>0.217996460670207</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
@@ -6874,19 +6874,19 @@
         <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>0.0000337990343787737</v>
+        <v>0.0337990343787737</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>0.00000265934666722365</v>
+        <v>0.00265934666722365</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
       </c>
       <c r="M4" t="n">
-        <v>0.0000109538940139369</v>
+        <v>0.0109538940139369</v>
       </c>
       <c r="N4" t="n">
         <v>0</v>
@@ -6895,19 +6895,19 @@
         <v>0</v>
       </c>
       <c r="P4" t="n">
-        <v>0.0221622814775544</v>
+        <v>22.1622814775544</v>
       </c>
       <c r="Q4" t="n">
         <v>0</v>
       </c>
       <c r="R4" t="n">
-        <v>0.000284198609196347</v>
+        <v>0.284198609196347</v>
       </c>
       <c r="S4" t="n">
         <v>0</v>
       </c>
       <c r="T4" t="n">
-        <v>0.000157109318162268</v>
+        <v>0.157109318162268</v>
       </c>
     </row>
     <row r="5">
@@ -6918,7 +6918,7 @@
         <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0000310025389670208</v>
+        <v>0.0310025389670208</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
@@ -6963,7 +6963,7 @@
         <v>0</v>
       </c>
       <c r="R5" t="n">
-        <v>0.00203382356276624</v>
+        <v>2.03382356276624</v>
       </c>
       <c r="S5" t="n">
         <v>0</v>
@@ -6977,61 +6977,61 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>0.00582588174954741</v>
+        <v>5.82588174954741</v>
       </c>
       <c r="C6" t="n">
         <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>0.000120092617282382</v>
+        <v>0.120092617282382</v>
       </c>
       <c r="E6" t="n">
-        <v>0.000789688400364426</v>
+        <v>0.789688400364426</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>0.00000940195316483307</v>
+        <v>0.00940195316483307</v>
       </c>
       <c r="H6" t="n">
-        <v>0.000471779809913899</v>
+        <v>0.471779809913899</v>
       </c>
       <c r="I6" t="n">
-        <v>0.000299703866991443</v>
+        <v>0.299703866991443</v>
       </c>
       <c r="J6" t="n">
-        <v>0.0000703739411962755</v>
+        <v>0.0703739411962755</v>
       </c>
       <c r="K6" t="n">
-        <v>0.0000300284561174004</v>
+        <v>0.0300284561174004</v>
       </c>
       <c r="L6" t="n">
-        <v>0.0000548139167916712</v>
+        <v>0.0548139167916712</v>
       </c>
       <c r="M6" t="n">
-        <v>0.0000250708787712242</v>
+        <v>0.0250708787712242</v>
       </c>
       <c r="N6" t="n">
-        <v>0.0000345941125625156</v>
+        <v>0.0345941125625156</v>
       </c>
       <c r="O6" t="n">
-        <v>0.000406420797016432</v>
+        <v>0.406420797016432</v>
       </c>
       <c r="P6" t="n">
-        <v>0.000448118518109753</v>
+        <v>0.448118518109753</v>
       </c>
       <c r="Q6" t="n">
         <v>0</v>
       </c>
       <c r="R6" t="n">
-        <v>0.000201162098619221</v>
+        <v>0.201162098619221</v>
       </c>
       <c r="S6" t="n">
         <v>0</v>
       </c>
       <c r="T6" t="n">
-        <v>0.00100498319568252</v>
+        <v>1.00498319568252</v>
       </c>
     </row>
     <row r="7">
@@ -7039,16 +7039,16 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>0.000010471395992783</v>
+        <v>0.010471395992783</v>
       </c>
       <c r="C7" t="n">
-        <v>0.0000023956507383607</v>
+        <v>0.0023956507383607</v>
       </c>
       <c r="D7" t="n">
-        <v>0.00000331895737562276</v>
+        <v>0.00331895737562276</v>
       </c>
       <c r="E7" t="n">
-        <v>0.000247036266507258</v>
+        <v>0.247036266507258</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
@@ -7057,43 +7057,43 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>0.00116551777200877</v>
+        <v>1.16551777200877</v>
       </c>
       <c r="I7" t="n">
-        <v>0.00270850567021767</v>
+        <v>2.70850567021767</v>
       </c>
       <c r="J7" t="n">
-        <v>0.0000164823178064961</v>
+        <v>0.0164823178064961</v>
       </c>
       <c r="K7" t="n">
-        <v>0.0000250421811163561</v>
+        <v>0.0250421811163561</v>
       </c>
       <c r="L7" t="n">
-        <v>0.0000289128352307716</v>
+        <v>0.0289128352307716</v>
       </c>
       <c r="M7" t="n">
-        <v>0.0000338709172206229</v>
+        <v>0.0338709172206229</v>
       </c>
       <c r="N7" t="n">
-        <v>0.0000715905940529838</v>
+        <v>0.0715905940529838</v>
       </c>
       <c r="O7" t="n">
-        <v>0.0048440635075255</v>
+        <v>4.8440635075255</v>
       </c>
       <c r="P7" t="n">
         <v>0</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.0000366117821529917</v>
+        <v>0.0366117821529917</v>
       </c>
       <c r="R7" t="n">
-        <v>0.00109624116128273</v>
+        <v>1.09624116128273</v>
       </c>
       <c r="S7" t="n">
         <v>0</v>
       </c>
       <c r="T7" t="n">
-        <v>0.0264526422238052</v>
+        <v>26.4526422238052</v>
       </c>
     </row>
     <row r="8">
@@ -7107,10 +7107,10 @@
         <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>0.000000281608504598295</v>
+        <v>0.000281608504598295</v>
       </c>
       <c r="E8" t="n">
-        <v>0.0000157253967172137</v>
+        <v>0.0157253967172137</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
@@ -7134,7 +7134,7 @@
         <v>0</v>
       </c>
       <c r="M8" t="n">
-        <v>0.0000000861542225815264</v>
+        <v>0.0000861542225815264</v>
       </c>
       <c r="N8" t="n">
         <v>0</v>
@@ -7149,13 +7149,13 @@
         <v>0</v>
       </c>
       <c r="R8" t="n">
-        <v>0.000140501056827768</v>
+        <v>0.140501056827768</v>
       </c>
       <c r="S8" t="n">
         <v>0</v>
       </c>
       <c r="T8" t="n">
-        <v>0.000031948430473861</v>
+        <v>0.031948430473861</v>
       </c>
     </row>
     <row r="9">
@@ -7172,7 +7172,7 @@
         <v>0</v>
       </c>
       <c r="E9" t="n">
-        <v>0.000247540054960441</v>
+        <v>0.247540054960441</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
@@ -7181,7 +7181,7 @@
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>0.000133934805096362</v>
+        <v>0.133934805096362</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
@@ -7193,16 +7193,16 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>0.0000383496633963707</v>
+        <v>0.0383496633963707</v>
       </c>
       <c r="M9" t="n">
-        <v>0.000000775388003233737</v>
+        <v>0.000775388003233737</v>
       </c>
       <c r="N9" t="n">
         <v>0</v>
       </c>
       <c r="O9" t="n">
-        <v>0.000445108147433827</v>
+        <v>0.445108147433827</v>
       </c>
       <c r="P9" t="n">
         <v>0</v>
@@ -7211,13 +7211,13 @@
         <v>0</v>
       </c>
       <c r="R9" t="n">
-        <v>0.000541671299072233</v>
+        <v>0.541671299072233</v>
       </c>
       <c r="S9" t="n">
         <v>0</v>
       </c>
       <c r="T9" t="n">
-        <v>0.00111647359806515</v>
+        <v>1.11647359806515</v>
       </c>
     </row>
     <row r="10">
@@ -7231,10 +7231,10 @@
         <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>0.00000050957729403501</v>
+        <v>0.00050957729403501</v>
       </c>
       <c r="E10" t="n">
-        <v>0.000958529501959773</v>
+        <v>0.958529501959773</v>
       </c>
       <c r="F10" t="n">
         <v>0</v>
@@ -7243,28 +7243,28 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>0.0173193851157586</v>
+        <v>17.3193851157586</v>
       </c>
       <c r="I10" t="n">
-        <v>0.00000181407246665735</v>
+        <v>0.00181407246665735</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>0.0253103319053011</v>
+        <v>25.3103319053011</v>
       </c>
       <c r="L10" t="n">
-        <v>0.0198848024299632</v>
+        <v>19.8848024299632</v>
       </c>
       <c r="M10" t="n">
-        <v>0.00367569605996432</v>
+        <v>3.67569605996432</v>
       </c>
       <c r="N10" t="n">
-        <v>0.00205402543339937</v>
+        <v>2.05402543339937</v>
       </c>
       <c r="O10" t="n">
-        <v>0.000748905657027272</v>
+        <v>0.748905657027272</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -7273,13 +7273,13 @@
         <v>0</v>
       </c>
       <c r="R10" t="n">
-        <v>0.00183909064197061</v>
+        <v>1.83909064197061</v>
       </c>
       <c r="S10" t="n">
         <v>0</v>
       </c>
       <c r="T10" t="n">
-        <v>0.0000384292531373384</v>
+        <v>0.0384292531373384</v>
       </c>
     </row>
     <row r="11">
@@ -7290,13 +7290,13 @@
         <v>0</v>
       </c>
       <c r="C11" t="n">
-        <v>0.0000111327299017938</v>
+        <v>0.0111327299017938</v>
       </c>
       <c r="D11" t="n">
         <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>0.000298206779394851</v>
+        <v>0.298206779394851</v>
       </c>
       <c r="F11" t="n">
         <v>0</v>
@@ -7305,10 +7305,10 @@
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>0.000385972878043653</v>
+        <v>0.385972878043653</v>
       </c>
       <c r="I11" t="n">
-        <v>0.00000229145995788297</v>
+        <v>0.00229145995788297</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -7320,13 +7320,13 @@
         <v>0</v>
       </c>
       <c r="M11" t="n">
-        <v>0.000823892830547136</v>
+        <v>0.823892830547136</v>
       </c>
       <c r="N11" t="n">
         <v>0</v>
       </c>
       <c r="O11" t="n">
-        <v>0.0000545695258519056</v>
+        <v>0.0545695258519056</v>
       </c>
       <c r="P11" t="n">
         <v>0</v>
@@ -7335,13 +7335,13 @@
         <v>0</v>
       </c>
       <c r="R11" t="n">
-        <v>0.000884231081570292</v>
+        <v>0.884231081570292</v>
       </c>
       <c r="S11" t="n">
         <v>0</v>
       </c>
       <c r="T11" t="n">
-        <v>0.0000235942450092223</v>
+        <v>0.0235942450092223</v>
       </c>
     </row>
     <row r="12">
@@ -7352,13 +7352,13 @@
         <v>0</v>
       </c>
       <c r="C12" t="n">
-        <v>0.0000169104758001931</v>
+        <v>0.0169104758001931</v>
       </c>
       <c r="D12" t="n">
-        <v>0.000000677201403914947</v>
+        <v>0.000677201403914947</v>
       </c>
       <c r="E12" t="n">
-        <v>0.0000697387158763389</v>
+        <v>0.0697387158763389</v>
       </c>
       <c r="F12" t="n">
         <v>0</v>
@@ -7367,7 +7367,7 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>0.000637694320246035</v>
+        <v>0.637694320246035</v>
       </c>
       <c r="I12" t="n">
         <v>0</v>
@@ -7376,19 +7376,19 @@
         <v>0</v>
       </c>
       <c r="K12" t="n">
-        <v>0.000168203676701896</v>
+        <v>0.168203676701896</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
       </c>
       <c r="M12" t="n">
-        <v>0.0000147077565692749</v>
+        <v>0.0147077565692749</v>
       </c>
       <c r="N12" t="n">
         <v>0</v>
       </c>
       <c r="O12" t="n">
-        <v>0.000182441399863088</v>
+        <v>0.182441399863087</v>
       </c>
       <c r="P12" t="n">
         <v>0</v>
@@ -7397,13 +7397,13 @@
         <v>0</v>
       </c>
       <c r="R12" t="n">
-        <v>0.000427128198485309</v>
+        <v>0.427128198485309</v>
       </c>
       <c r="S12" t="n">
         <v>0</v>
       </c>
       <c r="T12" t="n">
-        <v>0.0000183285765951469</v>
+        <v>0.0183285765951469</v>
       </c>
     </row>
     <row r="13">
@@ -7414,13 +7414,13 @@
         <v>0</v>
       </c>
       <c r="C13" t="n">
-        <v>0.000930921692800633</v>
+        <v>0.930921692800633</v>
       </c>
       <c r="D13" t="n">
         <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>0.00055812563634779</v>
+        <v>0.55812563634779</v>
       </c>
       <c r="F13" t="n">
         <v>0</v>
@@ -7453,19 +7453,19 @@
         <v>0</v>
       </c>
       <c r="P13" t="n">
-        <v>0.000682155127347941</v>
+        <v>0.682155127347941</v>
       </c>
       <c r="Q13" t="n">
         <v>0</v>
       </c>
       <c r="R13" t="n">
-        <v>0.0164842028607365</v>
+        <v>16.4842028607365</v>
       </c>
       <c r="S13" t="n">
         <v>0</v>
       </c>
       <c r="T13" t="n">
-        <v>0.0000722004149853025</v>
+        <v>0.0722004149853025</v>
       </c>
     </row>
     <row r="14">
@@ -7476,13 +7476,13 @@
         <v>0</v>
       </c>
       <c r="C14" t="n">
-        <v>0.00000267749200169725</v>
+        <v>0.00267749200169725</v>
       </c>
       <c r="D14" t="n">
-        <v>0.00000128064819948272</v>
+        <v>0.00128064819948272</v>
       </c>
       <c r="E14" t="n">
-        <v>0.000216413125531632</v>
+        <v>0.216413125531632</v>
       </c>
       <c r="F14" t="n">
         <v>0</v>
@@ -7491,28 +7491,28 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>0.0295080856410174</v>
+        <v>29.5080856410174</v>
       </c>
       <c r="I14" t="n">
-        <v>0.00000315075744208908</v>
+        <v>0.00315075744208908</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>0.000287209440060154</v>
+        <v>0.287209440060154</v>
       </c>
       <c r="L14" t="n">
-        <v>0.026643378448734</v>
+        <v>26.643378448734</v>
       </c>
       <c r="M14" t="n">
-        <v>0.0000267201167463562</v>
+        <v>0.0267201167463562</v>
       </c>
       <c r="N14" t="n">
         <v>0</v>
       </c>
       <c r="O14" t="n">
-        <v>0.00167414418490436</v>
+        <v>1.67414418490436</v>
       </c>
       <c r="P14" t="n">
         <v>0</v>
@@ -7521,13 +7521,13 @@
         <v>0</v>
       </c>
       <c r="R14" t="n">
-        <v>0.000663174316364996</v>
+        <v>0.663174316364996</v>
       </c>
       <c r="S14" t="n">
         <v>0</v>
       </c>
       <c r="T14" t="n">
-        <v>0.000120502796399032</v>
+        <v>0.120502796399032</v>
       </c>
     </row>
     <row r="15">
@@ -7541,10 +7541,10 @@
         <v>0</v>
       </c>
       <c r="D15" t="n">
-        <v>0.00000228639285876235</v>
+        <v>0.00228639285876235</v>
       </c>
       <c r="E15" t="n">
-        <v>0.0000351932219437871</v>
+        <v>0.0351932219437871</v>
       </c>
       <c r="F15" t="n">
         <v>0</v>
@@ -7553,7 +7553,7 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>0.00151127854544902</v>
+        <v>1.51127854544902</v>
       </c>
       <c r="I15" t="n">
         <v>0</v>
@@ -7568,7 +7568,7 @@
         <v>0</v>
       </c>
       <c r="M15" t="n">
-        <v>0.000298438227022407</v>
+        <v>0.298438227022407</v>
       </c>
       <c r="N15" t="n">
         <v>0</v>
@@ -7583,13 +7583,13 @@
         <v>0</v>
       </c>
       <c r="R15" t="n">
-        <v>0.000331386120727101</v>
+        <v>0.331386120727101</v>
       </c>
       <c r="S15" t="n">
         <v>0</v>
       </c>
       <c r="T15" t="n">
-        <v>0.0000497706927984238</v>
+        <v>0.0497706927984238</v>
       </c>
     </row>
     <row r="16">
@@ -7597,16 +7597,16 @@
         <v>15</v>
       </c>
       <c r="B16" t="n">
-        <v>0.00631324433155554</v>
+        <v>6.31324433155554</v>
       </c>
       <c r="C16" t="n">
-        <v>0.0000512951099272525</v>
+        <v>0.0512951099272525</v>
       </c>
       <c r="D16" t="n">
         <v>0</v>
       </c>
       <c r="E16" t="n">
-        <v>0.000118174377160938</v>
+        <v>0.118174377160938</v>
       </c>
       <c r="F16" t="n">
         <v>0</v>
@@ -7615,19 +7615,19 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>0.0000183645832047021</v>
+        <v>0.0183645832047021</v>
       </c>
       <c r="I16" t="n">
-        <v>0.00000773367735785501</v>
+        <v>0.00773367735785501</v>
       </c>
       <c r="J16" t="n">
-        <v>0.00000666700495543663</v>
+        <v>0.00666700495543663</v>
       </c>
       <c r="K16" t="n">
-        <v>0.00000797804000167096</v>
+        <v>0.00797804000167096</v>
       </c>
       <c r="L16" t="n">
-        <v>0.00000542115660576968</v>
+        <v>0.00542115660576968</v>
       </c>
       <c r="M16" t="n">
         <v>0</v>
@@ -7636,22 +7636,22 @@
         <v>0</v>
       </c>
       <c r="O16" t="n">
-        <v>0.0000154749401669583</v>
+        <v>0.0154749401669583</v>
       </c>
       <c r="P16" t="n">
         <v>0</v>
       </c>
       <c r="Q16" t="n">
-        <v>0.0000153987520469779</v>
+        <v>0.0153987520469779</v>
       </c>
       <c r="R16" t="n">
-        <v>0.0000179928522580203</v>
+        <v>0.0179928522580203</v>
       </c>
       <c r="S16" t="n">
         <v>0</v>
       </c>
       <c r="T16" t="n">
-        <v>0.0000181766823139717</v>
+        <v>0.0181766823139717</v>
       </c>
     </row>
     <row r="17">
@@ -7659,46 +7659,46 @@
         <v>16</v>
       </c>
       <c r="B17" t="n">
-        <v>0.000283490913087413</v>
+        <v>0.283490913087413</v>
       </c>
       <c r="C17" t="n">
-        <v>0.000502945734424078</v>
+        <v>0.502945734424078</v>
       </c>
       <c r="D17" t="n">
-        <v>0.0000180095343655005</v>
+        <v>0.0180095343655005</v>
       </c>
       <c r="E17" t="n">
-        <v>0.00036877314772999</v>
+        <v>0.36877314772999</v>
       </c>
       <c r="F17" t="n">
-        <v>0.000191483686750847</v>
+        <v>0.191483686750847</v>
       </c>
       <c r="G17" t="n">
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>0.000638327581735852</v>
+        <v>0.638327581735852</v>
       </c>
       <c r="I17" t="n">
-        <v>0.00000754272236136476</v>
+        <v>0.00754272236136476</v>
       </c>
       <c r="J17" t="n">
-        <v>0.0000333350247771831</v>
+        <v>0.0333350247771831</v>
       </c>
       <c r="K17" t="n">
-        <v>0.0000121886722247751</v>
+        <v>0.0121886722247751</v>
       </c>
       <c r="L17" t="n">
-        <v>0.0000379480962403877</v>
+        <v>0.0379480962403877</v>
       </c>
       <c r="M17" t="n">
-        <v>0.0000252431872163872</v>
+        <v>0.0252431872163872</v>
       </c>
       <c r="N17" t="n">
-        <v>0.0000293089009210202</v>
+        <v>0.0293089009210202</v>
       </c>
       <c r="O17" t="n">
-        <v>0.000638137664253255</v>
+        <v>0.638137664253255</v>
       </c>
       <c r="P17" t="n">
         <v>0</v>
@@ -7707,13 +7707,13 @@
         <v>0</v>
       </c>
       <c r="R17" t="n">
-        <v>0.000555076476598096</v>
+        <v>0.555076476598096</v>
       </c>
       <c r="S17" t="n">
-        <v>0.0000532561311923085</v>
+        <v>0.0532561311923085</v>
       </c>
       <c r="T17" t="n">
-        <v>0.00139823748964524</v>
+        <v>1.39823748964524</v>
       </c>
     </row>
     <row r="18">
@@ -7783,61 +7783,61 @@
         <v>18</v>
       </c>
       <c r="B19" t="n">
-        <v>0.00373511336888927</v>
+        <v>3.73511336888927</v>
       </c>
       <c r="C19" t="n">
-        <v>0.000056650093930647</v>
+        <v>0.056650093930647</v>
       </c>
       <c r="D19" t="n">
-        <v>0.0000857028548994144</v>
+        <v>0.0857028548994144</v>
       </c>
       <c r="E19" t="n">
-        <v>0.000165746401097222</v>
+        <v>0.165746401097222</v>
       </c>
       <c r="F19" t="n">
-        <v>0.0000172655325791669</v>
+        <v>0.0172655325791669</v>
       </c>
       <c r="G19" t="n">
-        <v>0.000011097387342098</v>
+        <v>0.011097387342098</v>
       </c>
       <c r="H19" t="n">
-        <v>0.0000797909477169815</v>
+        <v>0.0797909477169815</v>
       </c>
       <c r="I19" t="n">
-        <v>0.0000305527994384395</v>
+        <v>0.0305527994384395</v>
       </c>
       <c r="J19" t="n">
-        <v>0.0000222233498514554</v>
+        <v>0.0222233498514554</v>
       </c>
       <c r="K19" t="n">
-        <v>0.0000105265805577603</v>
+        <v>0.0105265805577603</v>
       </c>
       <c r="L19" t="n">
-        <v>0.0000102399624775649</v>
+        <v>0.0102399624775649</v>
       </c>
       <c r="M19" t="n">
-        <v>0.00000484925195673163</v>
+        <v>0.00484925195673163</v>
       </c>
       <c r="N19" t="n">
-        <v>0.00000264260582074772</v>
+        <v>0.00264260582074772</v>
       </c>
       <c r="O19" t="n">
-        <v>0.0000598635843300756</v>
+        <v>0.0598635843300756</v>
       </c>
       <c r="P19" t="n">
-        <v>0.000505519075954488</v>
+        <v>0.505519075954488</v>
       </c>
       <c r="Q19" t="n">
         <v>0</v>
       </c>
       <c r="R19" t="n">
-        <v>0.0000773632335858255</v>
+        <v>0.0773632335858255</v>
       </c>
       <c r="S19" t="n">
         <v>0</v>
       </c>
       <c r="T19" t="n">
-        <v>0.000268498457690785</v>
+        <v>0.268498457690785</v>
       </c>
     </row>
     <row r="20">
@@ -7854,7 +7854,7 @@
         <v>0</v>
       </c>
       <c r="E20" t="n">
-        <v>0.0000848523694718303</v>
+        <v>0.0848523694718303</v>
       </c>
       <c r="F20" t="n">
         <v>0</v>
@@ -7893,7 +7893,7 @@
         <v>0</v>
       </c>
       <c r="R20" t="n">
-        <v>0.000122552432809935</v>
+        <v>0.122552432809935</v>
       </c>
       <c r="S20" t="n">
         <v>0</v>
@@ -7989,7 +7989,7 @@
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>0.35495495015697</v>
+        <v>0.301136589133561</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
@@ -7998,28 +7998,28 @@
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>0.183329201302112</v>
+        <v>0.0176762048974383</v>
       </c>
       <c r="I2" t="n">
-        <v>0.0639699238242328</v>
+        <v>0.0204543303649114</v>
       </c>
       <c r="J2" t="n">
-        <v>0.0135192044929687</v>
+        <v>0.00222860614423661</v>
       </c>
       <c r="K2" t="n">
-        <v>0.0187262327816999</v>
+        <v>0.00515937586816421</v>
       </c>
       <c r="L2" t="n">
-        <v>0.000803134311965878</v>
+        <v>0.00012211540516365</v>
       </c>
       <c r="M2" t="n">
-        <v>0.024713954134815</v>
+        <v>0.0613019333921523</v>
       </c>
       <c r="N2" t="n">
-        <v>0.0096094757118099</v>
+        <v>0.0012211540516365</v>
       </c>
       <c r="O2" t="n">
-        <v>0.0830759945805131</v>
+        <v>0.00622788566334615</v>
       </c>
       <c r="P2" t="n">
         <v>0</v>
@@ -8028,13 +8028,13 @@
         <v>0</v>
       </c>
       <c r="R2" t="n">
-        <v>0.331997274591508</v>
+        <v>2.52079777994193</v>
       </c>
       <c r="S2" t="n">
         <v>0</v>
       </c>
       <c r="T2" t="n">
-        <v>0.379836965792243</v>
+        <v>0.229027442384425</v>
       </c>
     </row>
     <row r="3">
@@ -8042,31 +8042,31 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>3.82560088411553</v>
+        <v>17.6589052749834</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>0.036461596381084</v>
+        <v>0.766326395012086</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>0.183818385648889</v>
+        <v>0.348073960220642</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>0.0528773343997457</v>
+        <v>0.0235337454886021</v>
       </c>
       <c r="I3" t="n">
-        <v>0.020050274631476</v>
+        <v>0.029593332650338</v>
       </c>
       <c r="J3" t="n">
-        <v>0.00296311331352739</v>
+        <v>0.00225473010669242</v>
       </c>
       <c r="K3" t="n">
         <v>0</v>
@@ -8081,7 +8081,7 @@
         <v>0</v>
       </c>
       <c r="O3" t="n">
-        <v>0.0492754673737357</v>
+        <v>0.0170513964318614</v>
       </c>
       <c r="P3" t="n">
         <v>0</v>
@@ -8090,13 +8090,13 @@
         <v>0</v>
       </c>
       <c r="R3" t="n">
-        <v>0.113485643571536</v>
+        <v>3.9774848288371</v>
       </c>
       <c r="S3" t="n">
         <v>0</v>
       </c>
       <c r="T3" t="n">
-        <v>0.0939212971933633</v>
+        <v>0.261407771744652</v>
       </c>
     </row>
     <row r="4">
@@ -8104,7 +8104,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>0.183447867407093</v>
+        <v>0.0402901310507417</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
@@ -8113,7 +8113,7 @@
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>0.217996460670207</v>
+        <v>0.0406186743061064</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
@@ -8125,19 +8125,19 @@
         <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>0.0337990343787737</v>
+        <v>0.00237355739589991</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>0.00265934666722365</v>
+        <v>0.00016091914548474</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
       </c>
       <c r="M4" t="n">
-        <v>0.0109538940139369</v>
+        <v>0.00596741831172577</v>
       </c>
       <c r="N4" t="n">
         <v>0</v>
@@ -8146,19 +8146,19 @@
         <v>0</v>
       </c>
       <c r="P4" t="n">
-        <v>22.1622814775544</v>
+        <v>0.603185301956362</v>
       </c>
       <c r="Q4" t="n">
         <v>0</v>
       </c>
       <c r="R4" t="n">
-        <v>0.284198609196347</v>
+        <v>0.473926998345744</v>
       </c>
       <c r="S4" t="n">
         <v>0</v>
       </c>
       <c r="T4" t="n">
-        <v>0.157109318162268</v>
+        <v>0.0208055045182978</v>
       </c>
     </row>
     <row r="5">
@@ -8169,7 +8169,7 @@
         <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0310025389670208</v>
+        <v>0.00791667569287645</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
@@ -8214,7 +8214,7 @@
         <v>0</v>
       </c>
       <c r="R5" t="n">
-        <v>2.03382356276624</v>
+        <v>18.2023086321776</v>
       </c>
       <c r="S5" t="n">
         <v>0</v>
@@ -8228,61 +8228,61 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>5.82588174954741</v>
+        <v>14.2017935911534</v>
       </c>
       <c r="C6" t="n">
         <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>0.120092617282382</v>
+        <v>1.33294376735112</v>
       </c>
       <c r="E6" t="n">
-        <v>0.789688400364426</v>
+        <v>1.63315565711129</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>0.00940195316483307</v>
+        <v>0.0226982217096807</v>
       </c>
       <c r="H6" t="n">
-        <v>0.471779809913899</v>
+        <v>0.110886394581719</v>
       </c>
       <c r="I6" t="n">
-        <v>0.299703866991443</v>
+        <v>0.233605632612091</v>
       </c>
       <c r="J6" t="n">
-        <v>0.0703739411962755</v>
+        <v>0.0282797516382907</v>
       </c>
       <c r="K6" t="n">
-        <v>0.0300284561174004</v>
+        <v>0.0201679281420441</v>
       </c>
       <c r="L6" t="n">
-        <v>0.0548139167916712</v>
+        <v>0.0203167689401404</v>
       </c>
       <c r="M6" t="n">
-        <v>0.0250708787712242</v>
+        <v>0.151594352861048</v>
       </c>
       <c r="N6" t="n">
-        <v>0.0345941125625156</v>
+        <v>0.0107165374629312</v>
       </c>
       <c r="O6" t="n">
-        <v>0.406420797016432</v>
+        <v>0.0742715582500371</v>
       </c>
       <c r="P6" t="n">
-        <v>0.448118518109753</v>
+        <v>0.135370705868555</v>
       </c>
       <c r="Q6" t="n">
         <v>0</v>
       </c>
       <c r="R6" t="n">
-        <v>0.201162098619221</v>
+        <v>3.72332698477716</v>
       </c>
       <c r="S6" t="n">
         <v>0</v>
       </c>
       <c r="T6" t="n">
-        <v>1.00498319568252</v>
+        <v>1.4771705007064</v>
       </c>
     </row>
     <row r="7">
@@ -8290,16 +8290,16 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>0.010471395992783</v>
+        <v>0.0105733440509434</v>
       </c>
       <c r="C7" t="n">
-        <v>0.0023956507383607</v>
+        <v>0.00052404329115463</v>
       </c>
       <c r="D7" t="n">
-        <v>0.00331895737562276</v>
+        <v>0.0152589075953848</v>
       </c>
       <c r="E7" t="n">
-        <v>0.247036266507258</v>
+        <v>0.21162101139862</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
@@ -8308,43 +8308,43 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>1.16551777200877</v>
+        <v>0.113470785572953</v>
       </c>
       <c r="I7" t="n">
-        <v>2.70850567021767</v>
+        <v>0.874474122557326</v>
       </c>
       <c r="J7" t="n">
-        <v>0.0164823178064961</v>
+        <v>0.00274352075957424</v>
       </c>
       <c r="K7" t="n">
-        <v>0.0250421811163561</v>
+        <v>0.00696669316476155</v>
       </c>
       <c r="L7" t="n">
-        <v>0.0289128352307716</v>
+        <v>0.00443895493683922</v>
       </c>
       <c r="M7" t="n">
-        <v>0.0338709172206229</v>
+        <v>0.0848333610151495</v>
       </c>
       <c r="N7" t="n">
-        <v>0.0715905940529838</v>
+        <v>0.00918617063318116</v>
       </c>
       <c r="O7" t="n">
-        <v>4.8440635075255</v>
+        <v>0.36667617342849</v>
       </c>
       <c r="P7" t="n">
         <v>0</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.0366117821529917</v>
+        <v>0.0248458172159195</v>
       </c>
       <c r="R7" t="n">
-        <v>1.09624116128273</v>
+        <v>8.40460630353796</v>
       </c>
       <c r="S7" t="n">
         <v>0</v>
       </c>
       <c r="T7" t="n">
-        <v>26.4526422238052</v>
+        <v>16.1052375105995</v>
       </c>
     </row>
     <row r="8">
@@ -8358,10 +8358,10 @@
         <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>0.000281608504598295</v>
+        <v>0.0132984912861636</v>
       </c>
       <c r="E8" t="n">
-        <v>0.0157253967172137</v>
+        <v>0.138367635525083</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
@@ -8385,7 +8385,7 @@
         <v>0</v>
       </c>
       <c r="M8" t="n">
-        <v>0.0000861542225815264</v>
+        <v>0.0022164152143606</v>
       </c>
       <c r="N8" t="n">
         <v>0</v>
@@ -8400,13 +8400,13 @@
         <v>0</v>
       </c>
       <c r="R8" t="n">
-        <v>0.140501056827768</v>
+        <v>11.0643447500881</v>
       </c>
       <c r="S8" t="n">
         <v>0</v>
       </c>
       <c r="T8" t="n">
-        <v>0.031948430473861</v>
+        <v>0.199794000037362</v>
       </c>
     </row>
     <row r="9">
@@ -8423,7 +8423,7 @@
         <v>0</v>
       </c>
       <c r="E9" t="n">
-        <v>0.247540054960441</v>
+        <v>0.656789710428205</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
@@ -8432,7 +8432,7 @@
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>0.133934805096362</v>
+        <v>0.0403869817576873</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
@@ -8444,16 +8444,16 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>0.0383496633963707</v>
+        <v>0.0182362021648186</v>
       </c>
       <c r="M9" t="n">
-        <v>0.000775388003233737</v>
+        <v>0.00601508238944279</v>
       </c>
       <c r="N9" t="n">
         <v>0</v>
       </c>
       <c r="O9" t="n">
-        <v>0.445108147433827</v>
+        <v>0.10435690558192</v>
       </c>
       <c r="P9" t="n">
         <v>0</v>
@@ -8462,13 +8462,13 @@
         <v>0</v>
       </c>
       <c r="R9" t="n">
-        <v>0.541671299072233</v>
+        <v>12.8626330860848</v>
       </c>
       <c r="S9" t="n">
         <v>0</v>
       </c>
       <c r="T9" t="n">
-        <v>1.11647359806515</v>
+        <v>2.10537431380322</v>
       </c>
     </row>
     <row r="10">
@@ -8482,10 +8482,10 @@
         <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>0.00050957729403501</v>
+        <v>0.0140747882392551</v>
       </c>
       <c r="E10" t="n">
-        <v>0.958529501959773</v>
+        <v>4.93302808327682</v>
       </c>
       <c r="F10" t="n">
         <v>0</v>
@@ -8494,28 +8494,28 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>17.3193851157586</v>
+        <v>10.1299584460397</v>
       </c>
       <c r="I10" t="n">
-        <v>0.00181407246665735</v>
+        <v>0.00351869705981378</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>25.3103319053011</v>
+        <v>42.3021464422454</v>
       </c>
       <c r="L10" t="n">
-        <v>19.8848024299632</v>
+        <v>18.3409306324062</v>
       </c>
       <c r="M10" t="n">
-        <v>3.67569605996432</v>
+        <v>55.3081767482276</v>
       </c>
       <c r="N10" t="n">
-        <v>2.05402543339937</v>
+        <v>1.5834136769162</v>
       </c>
       <c r="O10" t="n">
-        <v>0.748905657027272</v>
+        <v>0.340572836473554</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -8524,13 +8524,13 @@
         <v>0</v>
       </c>
       <c r="R10" t="n">
-        <v>1.83909064197061</v>
+        <v>84.7080018504643</v>
       </c>
       <c r="S10" t="n">
         <v>0</v>
       </c>
       <c r="T10" t="n">
-        <v>0.0384292531373384</v>
+        <v>0.140562687810456</v>
       </c>
     </row>
     <row r="11">
@@ -8541,13 +8541,13 @@
         <v>0</v>
       </c>
       <c r="C11" t="n">
-        <v>0.0111327299017938</v>
+        <v>0.00875368277961119</v>
       </c>
       <c r="D11" t="n">
         <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>0.298206779394851</v>
+        <v>0.9182502429701</v>
       </c>
       <c r="F11" t="n">
         <v>0</v>
@@ -8556,10 +8556,10 @@
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>0.385972878043653</v>
+        <v>0.135072649472735</v>
       </c>
       <c r="I11" t="n">
-        <v>0.00229145995788297</v>
+        <v>0.00265934666722365</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -8571,13 +8571,13 @@
         <v>0</v>
       </c>
       <c r="M11" t="n">
-        <v>0.823892830547136</v>
+        <v>7.41747188544244</v>
       </c>
       <c r="N11" t="n">
         <v>0</v>
       </c>
       <c r="O11" t="n">
-        <v>0.0545695258519056</v>
+        <v>0.0148480188919987</v>
       </c>
       <c r="P11" t="n">
         <v>0</v>
@@ -8586,13 +8586,13 @@
         <v>0</v>
       </c>
       <c r="R11" t="n">
-        <v>0.884231081570292</v>
+        <v>24.368147542326</v>
       </c>
       <c r="S11" t="n">
         <v>0</v>
       </c>
       <c r="T11" t="n">
-        <v>0.0235942450092223</v>
+        <v>0.0516356477885926</v>
       </c>
     </row>
     <row r="12">
@@ -8603,13 +8603,13 @@
         <v>0</v>
       </c>
       <c r="C12" t="n">
-        <v>0.0169104758001931</v>
+        <v>0.0240940293589763</v>
       </c>
       <c r="D12" t="n">
-        <v>0.000677201403914947</v>
+        <v>0.0202791413771384</v>
       </c>
       <c r="E12" t="n">
-        <v>0.0697387158763389</v>
+        <v>0.389118574147468</v>
       </c>
       <c r="F12" t="n">
         <v>0</v>
@@ -8618,7 +8618,7 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>0.637694320246035</v>
+        <v>0.40437812607482</v>
       </c>
       <c r="I12" t="n">
         <v>0</v>
@@ -8627,19 +8627,19 @@
         <v>0</v>
       </c>
       <c r="K12" t="n">
-        <v>0.168203676701896</v>
+        <v>0.304789471391051</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
       </c>
       <c r="M12" t="n">
-        <v>0.0147077565692749</v>
+        <v>0.239936375699806</v>
       </c>
       <c r="N12" t="n">
         <v>0</v>
       </c>
       <c r="O12" t="n">
-        <v>0.182441399863087</v>
+        <v>0.0899510429401783</v>
       </c>
       <c r="P12" t="n">
         <v>0</v>
@@ -8648,13 +8648,13 @@
         <v>0</v>
       </c>
       <c r="R12" t="n">
-        <v>0.427128198485309</v>
+        <v>21.3294402736118</v>
       </c>
       <c r="S12" t="n">
         <v>0</v>
       </c>
       <c r="T12" t="n">
-        <v>0.0183285765951469</v>
+        <v>0.072683655232912</v>
       </c>
     </row>
     <row r="13">
@@ -8665,13 +8665,13 @@
         <v>0</v>
       </c>
       <c r="C13" t="n">
-        <v>0.930921692800633</v>
+        <v>0.0813049706247947</v>
       </c>
       <c r="D13" t="n">
         <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>0.55812563634779</v>
+        <v>0.190893141748496</v>
       </c>
       <c r="F13" t="n">
         <v>0</v>
@@ -8704,19 +8704,19 @@
         <v>0</v>
       </c>
       <c r="P13" t="n">
-        <v>0.682155127347941</v>
+        <v>0.0340801489040352</v>
       </c>
       <c r="Q13" t="n">
         <v>0</v>
       </c>
       <c r="R13" t="n">
-        <v>16.4842028607365</v>
+        <v>50.4591004674544</v>
       </c>
       <c r="S13" t="n">
         <v>0</v>
       </c>
       <c r="T13" t="n">
-        <v>0.0722004149853025</v>
+        <v>0.0175508459144652</v>
       </c>
     </row>
     <row r="14">
@@ -8727,13 +8727,13 @@
         <v>0</v>
       </c>
       <c r="C14" t="n">
-        <v>0.00267749200169725</v>
+        <v>0.0045645009631097</v>
       </c>
       <c r="D14" t="n">
-        <v>0.00128064819948272</v>
+        <v>0.0458852465238923</v>
       </c>
       <c r="E14" t="n">
-        <v>0.216413125531632</v>
+        <v>1.44478467327062</v>
       </c>
       <c r="F14" t="n">
         <v>0</v>
@@ -8742,28 +8742,28 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>29.5080856410174</v>
+        <v>22.3886369871603</v>
       </c>
       <c r="I14" t="n">
-        <v>0.00315075744208908</v>
+        <v>0.00792781746224317</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>0.287209440060154</v>
+        <v>0.622694026125282</v>
       </c>
       <c r="L14" t="n">
-        <v>26.643378448734</v>
+        <v>31.878714963251</v>
       </c>
       <c r="M14" t="n">
-        <v>0.0267201167463562</v>
+        <v>0.521554294258482</v>
       </c>
       <c r="N14" t="n">
         <v>0</v>
       </c>
       <c r="O14" t="n">
-        <v>1.67414418490436</v>
+        <v>0.987613866281263</v>
       </c>
       <c r="P14" t="n">
         <v>0</v>
@@ -8772,13 +8772,13 @@
         <v>0</v>
       </c>
       <c r="R14" t="n">
-        <v>0.663174316364996</v>
+        <v>39.6241926238625</v>
       </c>
       <c r="S14" t="n">
         <v>0</v>
       </c>
       <c r="T14" t="n">
-        <v>0.120502796399032</v>
+        <v>0.571763804852689</v>
       </c>
     </row>
     <row r="15">
@@ -8792,10 +8792,10 @@
         <v>0</v>
       </c>
       <c r="D15" t="n">
-        <v>0.00228639285876235</v>
+        <v>0.138867226235073</v>
       </c>
       <c r="E15" t="n">
-        <v>0.0351932219437871</v>
+        <v>0.398276091665401</v>
       </c>
       <c r="F15" t="n">
         <v>0</v>
@@ -8804,7 +8804,7 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>1.51127854544902</v>
+        <v>1.94373393202347</v>
       </c>
       <c r="I15" t="n">
         <v>0</v>
@@ -8819,7 +8819,7 @@
         <v>0</v>
       </c>
       <c r="M15" t="n">
-        <v>0.298438227022407</v>
+        <v>9.87464076758961</v>
       </c>
       <c r="N15" t="n">
         <v>0</v>
@@ -8834,13 +8834,13 @@
         <v>0</v>
       </c>
       <c r="R15" t="n">
-        <v>0.331386120727101</v>
+        <v>33.5639235163299</v>
       </c>
       <c r="S15" t="n">
         <v>0</v>
       </c>
       <c r="T15" t="n">
-        <v>0.0497706927984238</v>
+        <v>0.400312268003159</v>
       </c>
     </row>
     <row r="16">
@@ -8848,16 +8848,16 @@
         <v>15</v>
       </c>
       <c r="B16" t="n">
-        <v>6.31324433155554</v>
+        <v>50.9450890989689</v>
       </c>
       <c r="C16" t="n">
-        <v>0.0512951099272525</v>
+        <v>0.0896729744870533</v>
       </c>
       <c r="D16" t="n">
         <v>0</v>
       </c>
       <c r="E16" t="n">
-        <v>0.118174377160938</v>
+        <v>0.809027604987591</v>
       </c>
       <c r="F16" t="n">
         <v>0</v>
@@ -8866,19 +8866,19 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>0.0183645832047021</v>
+        <v>0.0142885508798052</v>
       </c>
       <c r="I16" t="n">
-        <v>0.00773367735785501</v>
+        <v>0.0199547003666245</v>
       </c>
       <c r="J16" t="n">
-        <v>0.00666700495543663</v>
+        <v>0.00886875571849978</v>
       </c>
       <c r="K16" t="n">
-        <v>0.00797804000167096</v>
+        <v>0.0177375114369996</v>
       </c>
       <c r="L16" t="n">
-        <v>0.00542115660576968</v>
+        <v>0.00665156678887484</v>
       </c>
       <c r="M16" t="n">
         <v>0</v>
@@ -8887,22 +8887,22 @@
         <v>0</v>
       </c>
       <c r="O16" t="n">
-        <v>0.0154749401669583</v>
+        <v>0.00936146436952755</v>
       </c>
       <c r="P16" t="n">
         <v>0</v>
       </c>
       <c r="Q16" t="n">
-        <v>0.0153987520469779</v>
+        <v>0.0835141163492063</v>
       </c>
       <c r="R16" t="n">
-        <v>0.0179928522580203</v>
+        <v>1.10243560667463</v>
       </c>
       <c r="S16" t="n">
         <v>0</v>
       </c>
       <c r="T16" t="n">
-        <v>0.0181766823139717</v>
+        <v>0.0884412028594839</v>
       </c>
     </row>
     <row r="17">
@@ -8910,46 +8910,46 @@
         <v>16</v>
       </c>
       <c r="B17" t="n">
-        <v>0.283490913087413</v>
+        <v>0.421807703564121</v>
       </c>
       <c r="C17" t="n">
-        <v>0.502945734424078</v>
+        <v>0.162118424942962</v>
       </c>
       <c r="D17" t="n">
-        <v>0.0180095343655005</v>
+        <v>0.122008991145082</v>
       </c>
       <c r="E17" t="n">
-        <v>0.36877314772999</v>
+        <v>0.465505637101562</v>
       </c>
       <c r="F17" t="n">
-        <v>0.191483686750847</v>
+        <v>0.116876073796089</v>
       </c>
       <c r="G17" t="n">
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>0.638327581735852</v>
+        <v>0.0915748794298156</v>
       </c>
       <c r="I17" t="n">
-        <v>0.00754272236136476</v>
+        <v>0.00358849973956122</v>
       </c>
       <c r="J17" t="n">
-        <v>0.0333350247771831</v>
+        <v>0.00817632852051925</v>
       </c>
       <c r="K17" t="n">
-        <v>0.0121886722247751</v>
+        <v>0.00499664520698398</v>
       </c>
       <c r="L17" t="n">
-        <v>0.0379480962403877</v>
+        <v>0.00858514494654521</v>
       </c>
       <c r="M17" t="n">
-        <v>0.0252431872163872</v>
+        <v>0.0931647210865832</v>
       </c>
       <c r="N17" t="n">
-        <v>0.0293089009210202</v>
+        <v>0.0055417337750186</v>
       </c>
       <c r="O17" t="n">
-        <v>0.638137664253255</v>
+        <v>0.0711794821758537</v>
       </c>
       <c r="P17" t="n">
         <v>0</v>
@@ -8958,13 +8958,13 @@
         <v>0</v>
       </c>
       <c r="R17" t="n">
-        <v>0.555076476598096</v>
+        <v>6.27092600690691</v>
       </c>
       <c r="S17" t="n">
-        <v>0.0532561311923085</v>
+        <v>0.00754039185781219</v>
       </c>
       <c r="T17" t="n">
-        <v>1.39823748964524</v>
+        <v>1.254430491237</v>
       </c>
     </row>
     <row r="18">
@@ -9034,61 +9034,61 @@
         <v>18</v>
       </c>
       <c r="B19" t="n">
-        <v>3.73511336888927</v>
+        <v>39.2513727890685</v>
       </c>
       <c r="C19" t="n">
-        <v>0.056650093930647</v>
+        <v>0.128969667104265</v>
       </c>
       <c r="D19" t="n">
-        <v>0.0857028548994144</v>
+        <v>4.10072210180776</v>
       </c>
       <c r="E19" t="n">
-        <v>0.165746401097222</v>
+        <v>1.47769723055285</v>
       </c>
       <c r="F19" t="n">
-        <v>0.0172655325791669</v>
+        <v>0.0744302556422625</v>
       </c>
       <c r="G19" t="n">
-        <v>0.011097387342098</v>
+        <v>0.115495224272476</v>
       </c>
       <c r="H19" t="n">
-        <v>0.0797909477169815</v>
+        <v>0.0808466569907334</v>
       </c>
       <c r="I19" t="n">
-        <v>0.0305527994384395</v>
+        <v>0.102662421575535</v>
       </c>
       <c r="J19" t="n">
-        <v>0.0222233498514554</v>
+        <v>0.0384984080908254</v>
       </c>
       <c r="K19" t="n">
-        <v>0.0105265805577603</v>
+        <v>0.0304779064052368</v>
       </c>
       <c r="L19" t="n">
-        <v>0.0102399624775649</v>
+        <v>0.0163618234386008</v>
       </c>
       <c r="M19" t="n">
-        <v>0.00484925195673163</v>
+        <v>0.126403106564877</v>
       </c>
       <c r="N19" t="n">
-        <v>0.00264260582074772</v>
+        <v>0.003529020741659</v>
       </c>
       <c r="O19" t="n">
-        <v>0.0598635843300756</v>
+        <v>0.0471605499112612</v>
       </c>
       <c r="P19" t="n">
-        <v>0.505519075954488</v>
+        <v>0.658322778353115</v>
       </c>
       <c r="Q19" t="n">
         <v>0</v>
       </c>
       <c r="R19" t="n">
-        <v>0.0773632335858255</v>
+        <v>6.17289891729644</v>
       </c>
       <c r="S19" t="n">
         <v>0</v>
       </c>
       <c r="T19" t="n">
-        <v>0.268498457690785</v>
+        <v>1.70130881754706</v>
       </c>
     </row>
     <row r="20">
@@ -9105,7 +9105,7 @@
         <v>0</v>
       </c>
       <c r="E20" t="n">
-        <v>0.0848523694718303</v>
+        <v>0.119388905003747</v>
       </c>
       <c r="F20" t="n">
         <v>0</v>
@@ -9144,7 +9144,7 @@
         <v>0</v>
       </c>
       <c r="R20" t="n">
-        <v>0.122552432809935</v>
+        <v>1.54324589674055</v>
       </c>
       <c r="S20" t="n">
         <v>0</v>

</xml_diff>